<commit_message>
[#1] added metrics from paper https://arxiv.org/pdf/2602.03593
</commit_message>
<xml_diff>
--- a/metrics and parser/final_list_of_metrics.xlsx
+++ b/metrics and parser/final_list_of_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DATA\DEV\UZH\DX-Metrics-Compass\metrics and parser\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66C6841A-BFC1-4029-87B2-EA96336792B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3628999B-BA60-4DEE-BF1A-78C2B5652A9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="0" windowWidth="38115" windowHeight="23385" tabRatio="562" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -51,7 +51,6 @@
     <author>tc={B51E8FD0-2567-4557-B58E-1C6A56D9BFA3}</author>
     <author>tc={E017DF4E-5656-4CEF-B774-80BA936A6D56}</author>
     <author>tc={8A92D669-9E50-4C59-82E5-97B139270D19}</author>
-    <author>tc={CD59760B-76A7-492D-B20B-A2D9CF3FBC59}</author>
     <author>tc={121DA4BD-014E-470E-AB44-B9514592A80F}</author>
     <author>tc={41A1A9E9-8671-443A-BC53-E9E6789FC6B2}</author>
     <author>tc={EF886BF9-B28D-42E1-9B64-C8A7E72E082A}</author>
@@ -118,15 +117,7 @@
     Lattice von NextJS Page Compilation Duration</t>
       </text>
     </comment>
-    <comment ref="B33" authorId="6" shapeId="0" xr:uid="{CD59760B-76A7-492D-B20B-A2D9CF3FBC59}">
-      <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    note that meta calls PRs/MRs diffs</t>
-      </text>
-    </comment>
-    <comment ref="H34" authorId="7" shapeId="0" xr:uid="{121DA4BD-014E-470E-AB44-B9514592A80F}">
+    <comment ref="H34" authorId="6" shapeId="0" xr:uid="{121DA4BD-014E-470E-AB44-B9514592A80F}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -134,7 +125,7 @@
     Nach Andres Input von Business zu Process verschoben.</t>
       </text>
     </comment>
-    <comment ref="C52" authorId="8" shapeId="0" xr:uid="{41A1A9E9-8671-443A-BC53-E9E6789FC6B2}">
+    <comment ref="C52" authorId="7" shapeId="0" xr:uid="{41A1A9E9-8671-443A-BC53-E9E6789FC6B2}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -142,7 +133,7 @@
     „Time to Restore Services“ ergänzt nach Andres Input.</t>
       </text>
     </comment>
-    <comment ref="B54" authorId="9" shapeId="0" xr:uid="{EF886BF9-B28D-42E1-9B64-C8A7E72E082A}">
+    <comment ref="B54" authorId="8" shapeId="0" xr:uid="{EF886BF9-B28D-42E1-9B64-C8A7E72E082A}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -150,7 +141,7 @@
     Name gekürzt nach Andres Input.</t>
       </text>
     </comment>
-    <comment ref="H58" authorId="10" shapeId="0" xr:uid="{7C21EAC9-D7DB-489B-AFEF-DEF502EE6ECC}">
+    <comment ref="H58" authorId="9" shapeId="0" xr:uid="{7C21EAC9-D7DB-489B-AFEF-DEF502EE6ECC}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -158,7 +149,7 @@
     Nach Andres Input von DevEx zu Business/HR gewechselt.</t>
       </text>
     </comment>
-    <comment ref="H61" authorId="11" shapeId="0" xr:uid="{917C3D96-4AA9-4D8E-8F4B-AEDAD8831587}">
+    <comment ref="H61" authorId="10" shapeId="0" xr:uid="{917C3D96-4AA9-4D8E-8F4B-AEDAD8831587}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -166,7 +157,7 @@
     Nach Andres Input von Business zu Quality verschoben.</t>
       </text>
     </comment>
-    <comment ref="J69" authorId="12" shapeId="0" xr:uid="{FDDDF671-A2B6-4958-A032-5551C66219BE}">
+    <comment ref="J69" authorId="11" shapeId="0" xr:uid="{FDDDF671-A2B6-4958-A032-5551C66219BE}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -174,7 +165,7 @@
     Von Knowledge Expansion zu Upskilling gewechselt.</t>
       </text>
     </comment>
-    <comment ref="C76" authorId="13" shapeId="0" xr:uid="{9ABBA003-3752-4178-8927-349ABCC5DB99}">
+    <comment ref="C76" authorId="12" shapeId="0" xr:uid="{9ABBA003-3752-4178-8927-349ABCC5DB99}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -182,7 +173,7 @@
     Nach Andres Kommentar zu einer Metrik zusammengefasst.</t>
       </text>
     </comment>
-    <comment ref="B77" authorId="14" shapeId="0" xr:uid="{80D5B2BD-D0F6-4AB8-8017-59A06F6C1C9C}">
+    <comment ref="B77" authorId="13" shapeId="0" xr:uid="{80D5B2BD-D0F6-4AB8-8017-59A06F6C1C9C}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -190,7 +181,7 @@
     Name angepasst nach Andres Input. Ursprünglich „Quality of Reviews of Work Contributed by Team Members“</t>
       </text>
     </comment>
-    <comment ref="C80" authorId="15" shapeId="0" xr:uid="{45640671-D7E4-4EA6-9099-D4E52C010FD7}">
+    <comment ref="C80" authorId="14" shapeId="0" xr:uid="{45640671-D7E4-4EA6-9099-D4E52C010FD7}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -198,7 +189,7 @@
     Nach Andres Input Availability hinzugefügt.</t>
       </text>
     </comment>
-    <comment ref="H85" authorId="16" shapeId="0" xr:uid="{EB733AEE-2F18-46F9-8A7B-0CA9B6B32FFC}">
+    <comment ref="H85" authorId="15" shapeId="0" xr:uid="{EB733AEE-2F18-46F9-8A7B-0CA9B6B32FFC}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -206,7 +197,7 @@
     Nach Andres Input von Business zu Process verschoben.</t>
       </text>
     </comment>
-    <comment ref="C90" authorId="17" shapeId="0" xr:uid="{C9FB5614-C3E5-4863-BFB7-AAB3A42EAACD}">
+    <comment ref="C90" authorId="16" shapeId="0" xr:uid="{C9FB5614-C3E5-4863-BFB7-AAB3A42EAACD}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -214,7 +205,7 @@
     Nach Andres Input. Production Incidents und System Uptime / Availability hinzugefügt.</t>
       </text>
     </comment>
-    <comment ref="F90" authorId="18" shapeId="0" xr:uid="{FCC3DA67-C366-4123-AE95-236C8FC56568}">
+    <comment ref="F90" authorId="17" shapeId="0" xr:uid="{FCC3DA67-C366-4123-AE95-236C8FC56568}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -222,7 +213,7 @@
     Nach Andres Input angepasst.</t>
       </text>
     </comment>
-    <comment ref="H91" authorId="19" shapeId="0" xr:uid="{24A13EBD-8030-4299-B820-E3DBAA902DCC}">
+    <comment ref="H91" authorId="18" shapeId="0" xr:uid="{24A13EBD-8030-4299-B820-E3DBAA902DCC}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -230,7 +221,7 @@
     Nach Andres Anregung von Business zu DevEx/Upskilling gewechselt.</t>
       </text>
     </comment>
-    <comment ref="C92" authorId="20" shapeId="0" xr:uid="{65177E12-2939-4BCC-8B47-DB95E81C94F5}">
+    <comment ref="C92" authorId="19" shapeId="0" xr:uid="{65177E12-2939-4BCC-8B47-DB95E81C94F5}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -243,7 +234,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1575" uniqueCount="705">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1610" uniqueCount="718">
   <si>
     <t>id</t>
   </si>
@@ -1663,9 +1654,6 @@
     <t>504; 214</t>
   </si>
   <si>
-    <t>504; 11; 96; 214</t>
-  </si>
-  <si>
     <t>https://doi.org/10.1145/3454122.3454124</t>
   </si>
   <si>
@@ -1957,9 +1945,6 @@
     <t>105; 501; 131; 232</t>
   </si>
   <si>
-    <t>506; 9; 13; 15; 45; 87; 233; 235; 236; 237; 238; 232</t>
-  </si>
-  <si>
     <t>508; 237; 232</t>
   </si>
   <si>
@@ -2360,6 +2345,51 @@
   </si>
   <si>
     <t>Human-equivalent hours of work completed by agents</t>
+  </si>
+  <si>
+    <t>513</t>
+  </si>
+  <si>
+    <t>https://arxiv.org/pdf/2602.03593</t>
+  </si>
+  <si>
+    <t>Chen (2026)</t>
+  </si>
+  <si>
+    <t>504; 11; 96; 214; 513</t>
+  </si>
+  <si>
+    <t>506; 9; 13; 15; 45; 87; 233; 235; 236; 237; 238; 232; 513</t>
+  </si>
+  <si>
+    <t>Self-sufficiency</t>
+  </si>
+  <si>
+    <t>Degree to which AI reduces context-switching and reliance on external resources.</t>
+  </si>
+  <si>
+    <t>Code ownership</t>
+  </si>
+  <si>
+    <t>149</t>
+  </si>
+  <si>
+    <t>Whether developers maintain deep understanding of and accountability for AI-assisted code.</t>
+  </si>
+  <si>
+    <t>506; 512</t>
+  </si>
+  <si>
+    <t>Technical expertise development; Skill development</t>
+  </si>
+  <si>
+    <t>38</t>
+  </si>
+  <si>
+    <t>Ease of peer review</t>
+  </si>
+  <si>
+    <t>Perceived ease and effort to perform a PR.</t>
   </si>
 </sst>
 </file>
@@ -2923,7 +2953,6 @@
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
 <personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <person displayName="Patrick Meyer" id="{2315245B-EC09-46AB-A06E-DE769C358132}" userId="S::patrick.meyer@oec.uzh.ch::70537bee-da28-4c70-a2c9-3c1febc86743" providerId="AD"/>
-  <person displayName="André Meyer" id="{9D9142B8-11C7-4802-A1A1-66D498664CB5}" userId="S::andre.meyer@access.uzh.ch::3b573077-43ef-44d1-acd0-87895ce1f23f" providerId="AD"/>
 </personList>
 </file>
 
@@ -3212,9 +3241,6 @@
   <threadedComment ref="D29" dT="2025-05-23T09:41:06.69" personId="{2315245B-EC09-46AB-A06E-DE769C358132}" id="{8A92D669-9E50-4C59-82E5-97B139270D19}">
     <text>Lattice von NextJS Page Compilation Duration</text>
   </threadedComment>
-  <threadedComment ref="B33" dT="2025-04-03T11:15:23.43" personId="{9D9142B8-11C7-4802-A1A1-66D498664CB5}" id="{CD59760B-76A7-492D-B20B-A2D9CF3FBC59}">
-    <text>note that meta calls PRs/MRs diffs</text>
-  </threadedComment>
   <threadedComment ref="H34" dT="2025-06-02T18:38:57.61" personId="{2315245B-EC09-46AB-A06E-DE769C358132}" id="{121DA4BD-014E-470E-AB44-B9514592A80F}">
     <text>Nach Andres Input von Business zu Process verschoben.</text>
   </threadedComment>
@@ -3322,19 +3348,19 @@
         <v>10</v>
       </c>
       <c r="N1" s="6" t="s">
+        <v>530</v>
+      </c>
+      <c r="O1" s="1" t="s">
         <v>531</v>
       </c>
-      <c r="O1" s="1" t="s">
-        <v>532</v>
-      </c>
       <c r="P1" s="1" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="Q1" s="22" t="s">
-        <v>635</v>
+        <v>633</v>
       </c>
       <c r="R1" s="22" t="s">
-        <v>626</v>
+        <v>624</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="120" x14ac:dyDescent="0.25">
@@ -3348,16 +3374,16 @@
         <v>15</v>
       </c>
       <c r="D2" s="19" t="s">
-        <v>634</v>
+        <v>632</v>
       </c>
       <c r="E2" s="20" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="F2" s="8" t="s">
         <v>16</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H2" s="7" t="s">
         <v>17</v>
@@ -3393,7 +3419,7 @@
         <v>22</v>
       </c>
       <c r="Q2" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R2" s="19" t="s">
         <v>11</v>
@@ -3419,7 +3445,7 @@
         <v>22</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H3" s="7" t="s">
         <v>23</v>
@@ -3455,7 +3481,7 @@
         <v>1</v>
       </c>
       <c r="Q3" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R3" s="19" t="s">
         <v>11</v>
@@ -3472,19 +3498,19 @@
         <v>275</v>
       </c>
       <c r="D4" s="19" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="E4" s="20" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="F4" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="I4" s="7">
         <f>VLOOKUP(H4,cardsort_group_IDs!A:B,2,0)</f>
@@ -3517,7 +3543,7 @@
         <v>8</v>
       </c>
       <c r="Q4" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R4" s="19" t="s">
         <v>11</v>
@@ -3534,16 +3560,16 @@
         <v>11</v>
       </c>
       <c r="D5" s="19" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="E5" s="20" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="F5" s="10" t="s">
         <v>29</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H5" s="7" t="s">
         <v>17</v>
@@ -3579,7 +3605,7 @@
         <v>3</v>
       </c>
       <c r="Q5" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R5" s="19" t="s">
         <v>11</v>
@@ -3599,16 +3625,16 @@
         <v>446</v>
       </c>
       <c r="E6" s="20" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="F6" s="8" t="s">
         <v>32</v>
       </c>
       <c r="G6" s="7" t="s">
+        <v>533</v>
+      </c>
+      <c r="H6" s="7" t="s">
         <v>534</v>
-      </c>
-      <c r="H6" s="7" t="s">
-        <v>535</v>
       </c>
       <c r="I6" s="7">
         <f>VLOOKUP(H6,cardsort_group_IDs!A:B,2,0)</f>
@@ -3641,7 +3667,7 @@
         <v>4</v>
       </c>
       <c r="Q6" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R6" s="19" t="s">
         <v>11</v>
@@ -3667,7 +3693,7 @@
         <v>35</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H7" s="7" t="s">
         <v>12</v>
@@ -3703,7 +3729,7 @@
         <v>1</v>
       </c>
       <c r="Q7" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R7" s="19" t="s">
         <v>11</v>
@@ -3720,16 +3746,16 @@
         <v>11</v>
       </c>
       <c r="D8" s="20" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="E8" s="20" t="s">
-        <v>701</v>
+        <v>699</v>
       </c>
       <c r="F8" s="8" t="s">
         <v>37</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H8" s="7" t="s">
         <v>38</v>
@@ -3791,7 +3817,7 @@
         <v>42</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H9" s="7" t="s">
         <v>38</v>
@@ -3827,7 +3853,7 @@
         <v>1</v>
       </c>
       <c r="Q9" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R9" s="19" t="s">
         <v>11</v>
@@ -3853,7 +3879,7 @@
         <v>45</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H10" s="7" t="s">
         <v>38</v>
@@ -3889,7 +3915,7 @@
         <v>2</v>
       </c>
       <c r="Q10" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R10" s="19" t="s">
         <v>11</v>
@@ -3915,7 +3941,7 @@
         <v>47</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H11" s="7" t="s">
         <v>17</v>
@@ -3951,7 +3977,7 @@
         <v>3</v>
       </c>
       <c r="Q11" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R11" s="19" t="s">
         <v>11</v>
@@ -3977,7 +4003,7 @@
         <v>49</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H12" s="7" t="s">
         <v>38</v>
@@ -4013,7 +4039,7 @@
         <v>6</v>
       </c>
       <c r="Q12" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R12" s="19" t="s">
         <v>11</v>
@@ -4030,16 +4056,16 @@
         <v>52</v>
       </c>
       <c r="D13" s="20" t="s">
+        <v>549</v>
+      </c>
+      <c r="E13" s="20" t="s">
         <v>550</v>
-      </c>
-      <c r="E13" s="20" t="s">
-        <v>551</v>
       </c>
       <c r="F13" s="8" t="s">
         <v>53</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H13" s="7" t="s">
         <v>54</v>
@@ -4075,7 +4101,7 @@
         <v>8</v>
       </c>
       <c r="Q13" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R13" s="19" t="s">
         <v>11</v>
@@ -4089,10 +4115,10 @@
         <v>55</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
       <c r="D14" s="19" t="s">
-        <v>687</v>
+        <v>685</v>
       </c>
       <c r="E14" s="20">
         <v>131</v>
@@ -4101,7 +4127,7 @@
         <v>56</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H14" s="7" t="s">
         <v>38</v>
@@ -4154,16 +4180,16 @@
         <v>277</v>
       </c>
       <c r="D15" s="19" t="s">
-        <v>632</v>
+        <v>630</v>
       </c>
       <c r="E15" s="20" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="F15" s="8" t="s">
         <v>58</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H15" s="7" t="s">
         <v>59</v>
@@ -4199,7 +4225,7 @@
         <v>26</v>
       </c>
       <c r="Q15" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R15" s="19" t="s">
         <v>11</v>
@@ -4219,16 +4245,16 @@
         <v>11</v>
       </c>
       <c r="E16" s="20" t="s">
-        <v>472</v>
+        <v>706</v>
       </c>
       <c r="F16" s="8" t="s">
         <v>62</v>
       </c>
       <c r="G16" s="7" t="s">
+        <v>533</v>
+      </c>
+      <c r="H16" s="7" t="s">
         <v>534</v>
-      </c>
-      <c r="H16" s="7" t="s">
-        <v>535</v>
       </c>
       <c r="I16" s="7">
         <f>VLOOKUP(H16,cardsort_group_IDs!A:B,2,0)</f>
@@ -4254,14 +4280,14 @@
       </c>
       <c r="O16" s="7">
         <f t="shared" si="1"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="P16" s="7">
         <f t="shared" si="2"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q16" s="19" t="s">
-        <v>633</v>
+        <v>136</v>
       </c>
       <c r="R16" s="19" t="s">
         <v>11</v>
@@ -4287,7 +4313,7 @@
         <v>66</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H17" s="7" t="s">
         <v>17</v>
@@ -4323,7 +4349,7 @@
         <v>3</v>
       </c>
       <c r="Q17" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R17" s="19" t="s">
         <v>11</v>
@@ -4349,7 +4375,7 @@
         <v>69</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H18" s="7" t="s">
         <v>54</v>
@@ -4385,7 +4411,7 @@
         <v>2</v>
       </c>
       <c r="Q18" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R18" s="19" t="s">
         <v>11</v>
@@ -4411,7 +4437,7 @@
         <v>73</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H19" s="7" t="s">
         <v>12</v>
@@ -4447,7 +4473,7 @@
         <v>1</v>
       </c>
       <c r="Q19" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R19" s="19" t="s">
         <v>11</v>
@@ -4467,13 +4493,13 @@
         <v>11</v>
       </c>
       <c r="E20" s="20" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="F20" s="8" t="s">
         <v>76</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="H20" s="7" t="s">
         <v>77</v>
@@ -4509,7 +4535,7 @@
         <v>3</v>
       </c>
       <c r="Q20" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R20" s="19" t="s">
         <v>11</v>
@@ -4535,7 +4561,7 @@
         <v>79</v>
       </c>
       <c r="G21" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H21" s="7" t="s">
         <v>77</v>
@@ -4571,7 +4597,7 @@
         <v>3</v>
       </c>
       <c r="Q21" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R21" s="19" t="s">
         <v>11</v>
@@ -4585,10 +4611,10 @@
         <v>30</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>663</v>
+        <v>661</v>
       </c>
       <c r="D22" s="20" t="s">
-        <v>664</v>
+        <v>662</v>
       </c>
       <c r="E22" s="20" t="s">
         <v>456</v>
@@ -4597,7 +4623,7 @@
         <v>80</v>
       </c>
       <c r="G22" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H22" s="7" t="s">
         <v>17</v>
@@ -4659,10 +4685,10 @@
         <v>83</v>
       </c>
       <c r="G23" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="I23" s="7">
         <f>VLOOKUP(H23,cardsort_group_IDs!A:B,2,0)</f>
@@ -4695,7 +4721,7 @@
         <v>2</v>
       </c>
       <c r="Q23" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R23" s="19" t="s">
         <v>11</v>
@@ -4721,7 +4747,7 @@
         <v>85</v>
       </c>
       <c r="G24" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H24" s="7" t="s">
         <v>38</v>
@@ -4757,7 +4783,7 @@
         <v>1</v>
       </c>
       <c r="Q24" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R24" s="19" t="s">
         <v>11</v>
@@ -4774,16 +4800,16 @@
         <v>11</v>
       </c>
       <c r="D25" s="20" t="s">
-        <v>669</v>
+        <v>667</v>
       </c>
       <c r="E25" s="20" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="F25" s="8" t="s">
         <v>87</v>
       </c>
       <c r="G25" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H25" s="7" t="s">
         <v>77</v>
@@ -4839,13 +4865,13 @@
         <v>170</v>
       </c>
       <c r="E26" s="20" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="F26" s="8" t="s">
         <v>89</v>
       </c>
       <c r="G26" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H26" s="7" t="s">
         <v>38</v>
@@ -4881,7 +4907,7 @@
         <v>4</v>
       </c>
       <c r="Q26" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R26" s="19" t="s">
         <v>11</v>
@@ -4907,7 +4933,7 @@
         <v>93</v>
       </c>
       <c r="G27" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H27" s="7" t="s">
         <v>77</v>
@@ -4943,7 +4969,7 @@
         <v>2</v>
       </c>
       <c r="Q27" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R27" s="19" t="s">
         <v>11</v>
@@ -4969,7 +4995,7 @@
         <v>95</v>
       </c>
       <c r="G28" s="7" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="H28" s="7" t="s">
         <v>17</v>
@@ -5005,7 +5031,7 @@
         <v>3</v>
       </c>
       <c r="Q28" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R28" s="19" t="s">
         <v>11</v>
@@ -5022,16 +5048,16 @@
         <v>282</v>
       </c>
       <c r="D29" s="20" t="s">
+        <v>551</v>
+      </c>
+      <c r="E29" s="20" t="s">
         <v>552</v>
-      </c>
-      <c r="E29" s="20" t="s">
-        <v>553</v>
       </c>
       <c r="F29" s="8" t="s">
         <v>98</v>
       </c>
       <c r="G29" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H29" s="7" t="s">
         <v>23</v>
@@ -5067,7 +5093,7 @@
         <v>8</v>
       </c>
       <c r="Q29" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R29" s="19" t="s">
         <v>11</v>
@@ -5093,10 +5119,10 @@
         <v>100</v>
       </c>
       <c r="G30" s="7" t="s">
+        <v>533</v>
+      </c>
+      <c r="H30" s="7" t="s">
         <v>534</v>
-      </c>
-      <c r="H30" s="7" t="s">
-        <v>535</v>
       </c>
       <c r="I30" s="7">
         <f>VLOOKUP(H30,cardsort_group_IDs!A:B,2,0)</f>
@@ -5129,7 +5155,7 @@
         <v>3</v>
       </c>
       <c r="Q30" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R30" s="19" t="s">
         <v>11</v>
@@ -5143,22 +5169,22 @@
         <v>102</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>674</v>
+        <v>672</v>
       </c>
       <c r="D31" s="20" t="s">
-        <v>675</v>
+        <v>673</v>
       </c>
       <c r="E31" s="20" t="s">
-        <v>696</v>
+        <v>694</v>
       </c>
       <c r="F31" s="8" t="s">
         <v>103</v>
       </c>
       <c r="G31" s="7" t="s">
+        <v>533</v>
+      </c>
+      <c r="H31" s="7" t="s">
         <v>534</v>
-      </c>
-      <c r="H31" s="7" t="s">
-        <v>535</v>
       </c>
       <c r="I31" s="7">
         <f>VLOOKUP(H31,cardsort_group_IDs!A:B,2,0)</f>
@@ -5217,7 +5243,7 @@
         <v>106</v>
       </c>
       <c r="G32" s="7" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="H32" s="7" t="s">
         <v>12</v>
@@ -5253,7 +5279,7 @@
         <v>1</v>
       </c>
       <c r="Q32" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R32" s="19" t="s">
         <v>11</v>
@@ -5270,7 +5296,7 @@
         <v>283</v>
       </c>
       <c r="D33" s="19" t="s">
-        <v>685</v>
+        <v>683</v>
       </c>
       <c r="E33" s="20" t="s">
         <v>468</v>
@@ -5279,7 +5305,7 @@
         <v>108</v>
       </c>
       <c r="G33" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H33" s="7" t="s">
         <v>17</v>
@@ -5341,7 +5367,7 @@
         <v>110</v>
       </c>
       <c r="G34" s="7" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="H34" s="7" t="s">
         <v>17</v>
@@ -5377,7 +5403,7 @@
         <v>3</v>
       </c>
       <c r="Q34" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R34" s="19" t="s">
         <v>11</v>
@@ -5394,19 +5420,19 @@
         <v>111</v>
       </c>
       <c r="D35" s="20" t="s">
+        <v>541</v>
+      </c>
+      <c r="E35" s="20" t="s">
         <v>542</v>
-      </c>
-      <c r="E35" s="20" t="s">
-        <v>543</v>
       </c>
       <c r="F35" s="8" t="s">
         <v>112</v>
       </c>
       <c r="G35" s="7" t="s">
+        <v>533</v>
+      </c>
+      <c r="H35" s="7" t="s">
         <v>534</v>
-      </c>
-      <c r="H35" s="7" t="s">
-        <v>535</v>
       </c>
       <c r="I35" s="7">
         <f>VLOOKUP(H35,cardsort_group_IDs!A:B,2,0)</f>
@@ -5465,10 +5491,10 @@
         <v>114</v>
       </c>
       <c r="G36" s="7" t="s">
+        <v>533</v>
+      </c>
+      <c r="H36" s="7" t="s">
         <v>534</v>
-      </c>
-      <c r="H36" s="7" t="s">
-        <v>535</v>
       </c>
       <c r="I36" s="7">
         <f>VLOOKUP(H36,cardsort_group_IDs!A:B,2,0)</f>
@@ -5501,7 +5527,7 @@
         <v>6</v>
       </c>
       <c r="Q36" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R36" s="19" t="s">
         <v>11</v>
@@ -5521,13 +5547,13 @@
         <v>11</v>
       </c>
       <c r="E37" s="20" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="F37" s="8" t="s">
         <v>116</v>
       </c>
       <c r="G37" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H37" s="7" t="s">
         <v>38</v>
@@ -5563,7 +5589,7 @@
         <v>2</v>
       </c>
       <c r="Q37" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R37" s="19" t="s">
         <v>11</v>
@@ -5589,10 +5615,10 @@
         <v>118</v>
       </c>
       <c r="G38" s="7" t="s">
+        <v>533</v>
+      </c>
+      <c r="H38" s="7" t="s">
         <v>534</v>
-      </c>
-      <c r="H38" s="7" t="s">
-        <v>535</v>
       </c>
       <c r="I38" s="7">
         <f>VLOOKUP(H38,cardsort_group_IDs!A:B,2,0)</f>
@@ -5625,7 +5651,7 @@
         <v>3</v>
       </c>
       <c r="Q38" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R38" s="19" t="s">
         <v>11</v>
@@ -5639,19 +5665,19 @@
         <v>120</v>
       </c>
       <c r="C39" s="8" t="s">
-        <v>612</v>
+        <v>610</v>
       </c>
       <c r="D39" s="20" t="s">
         <v>442</v>
       </c>
       <c r="E39" s="20" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="F39" s="8" t="s">
         <v>122</v>
       </c>
       <c r="G39" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H39" s="7" t="s">
         <v>23</v>
@@ -5713,7 +5739,7 @@
         <v>125</v>
       </c>
       <c r="G40" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H40" s="7" t="s">
         <v>23</v>
@@ -5749,7 +5775,7 @@
         <v>2</v>
       </c>
       <c r="Q40" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R40" s="19" t="s">
         <v>11</v>
@@ -5775,7 +5801,7 @@
         <v>128</v>
       </c>
       <c r="G41" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H41" s="7" t="s">
         <v>54</v>
@@ -5837,10 +5863,10 @@
         <v>131</v>
       </c>
       <c r="G42" s="7" t="s">
+        <v>533</v>
+      </c>
+      <c r="H42" s="7" t="s">
         <v>534</v>
-      </c>
-      <c r="H42" s="7" t="s">
-        <v>535</v>
       </c>
       <c r="I42" s="7">
         <f>VLOOKUP(H42,cardsort_group_IDs!A:B,2,0)</f>
@@ -5873,7 +5899,7 @@
         <v>2</v>
       </c>
       <c r="Q42" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R42" s="19" t="s">
         <v>11</v>
@@ -5899,7 +5925,7 @@
         <v>133</v>
       </c>
       <c r="G43" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H43" s="7" t="s">
         <v>17</v>
@@ -5935,7 +5961,7 @@
         <v>1</v>
       </c>
       <c r="Q43" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R43" s="19" t="s">
         <v>11</v>
@@ -5961,7 +5987,7 @@
         <v>135</v>
       </c>
       <c r="G44" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H44" s="7" t="s">
         <v>17</v>
@@ -5997,7 +6023,7 @@
         <v>1</v>
       </c>
       <c r="Q44" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R44" s="19" t="s">
         <v>11</v>
@@ -6017,16 +6043,16 @@
         <v>446</v>
       </c>
       <c r="E45" s="20" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="F45" s="8" t="s">
         <v>137</v>
       </c>
       <c r="G45" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H45" s="7" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="I45" s="7">
         <f>VLOOKUP(H45,cardsort_group_IDs!A:B,2,0)</f>
@@ -6059,7 +6085,7 @@
         <v>4</v>
       </c>
       <c r="Q45" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R45" s="19" t="s">
         <v>11</v>
@@ -6085,7 +6111,7 @@
         <v>140</v>
       </c>
       <c r="G46" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H46" s="7" t="s">
         <v>12</v>
@@ -6121,7 +6147,7 @@
         <v>1</v>
       </c>
       <c r="Q46" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R46" s="19" t="s">
         <v>11</v>
@@ -6138,19 +6164,19 @@
         <v>285</v>
       </c>
       <c r="D47" s="19" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="E47" s="20" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="F47" s="8" t="s">
         <v>142</v>
       </c>
       <c r="G47" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H47" s="7" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="I47" s="7">
         <f>VLOOKUP(H47,cardsort_group_IDs!A:B,2,0)</f>
@@ -6209,10 +6235,10 @@
         <v>144</v>
       </c>
       <c r="G48" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H48" s="7" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="I48" s="7">
         <f>VLOOKUP(H48,cardsort_group_IDs!A:B,2,0)</f>
@@ -6262,16 +6288,16 @@
         <v>147</v>
       </c>
       <c r="D49" s="20" t="s">
-        <v>670</v>
+        <v>668</v>
       </c>
       <c r="E49" s="20" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="F49" s="8" t="s">
         <v>148</v>
       </c>
       <c r="G49" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H49" s="7" t="s">
         <v>17</v>
@@ -6307,7 +6333,7 @@
         <v>11</v>
       </c>
       <c r="Q49" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R49" s="19" t="s">
         <v>11</v>
@@ -6324,7 +6350,7 @@
         <v>287</v>
       </c>
       <c r="D50" s="19" t="s">
-        <v>688</v>
+        <v>686</v>
       </c>
       <c r="E50" s="20" t="s">
         <v>465</v>
@@ -6333,7 +6359,7 @@
         <v>151</v>
       </c>
       <c r="G50" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H50" s="7" t="s">
         <v>38</v>
@@ -6395,7 +6421,7 @@
         <v>153</v>
       </c>
       <c r="G51" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H51" s="7" t="s">
         <v>23</v>
@@ -6431,7 +6457,7 @@
         <v>1</v>
       </c>
       <c r="Q51" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R51" s="19" t="s">
         <v>11</v>
@@ -6448,16 +6474,16 @@
         <v>288</v>
       </c>
       <c r="D52" s="20" t="s">
-        <v>671</v>
+        <v>669</v>
       </c>
       <c r="E52" s="20" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="F52" s="8" t="s">
         <v>155</v>
       </c>
       <c r="G52" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H52" s="7" t="s">
         <v>23</v>
@@ -6493,7 +6519,7 @@
         <v>16</v>
       </c>
       <c r="Q52" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R52" s="19" t="s">
         <v>11</v>
@@ -6519,7 +6545,7 @@
         <v>157</v>
       </c>
       <c r="G53" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H53" s="7" t="s">
         <v>54</v>
@@ -6555,7 +6581,7 @@
         <v>1</v>
       </c>
       <c r="Q53" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R53" s="19" t="s">
         <v>11</v>
@@ -6581,7 +6607,7 @@
         <v>159</v>
       </c>
       <c r="G54" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H54" s="7" t="s">
         <v>54</v>
@@ -6617,7 +6643,7 @@
         <v>3</v>
       </c>
       <c r="Q54" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R54" s="19" t="s">
         <v>11</v>
@@ -6643,7 +6669,7 @@
         <v>161</v>
       </c>
       <c r="G55" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H55" s="7" t="s">
         <v>77</v>
@@ -6679,7 +6705,7 @@
         <v>3</v>
       </c>
       <c r="Q55" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R55" s="19" t="s">
         <v>11</v>
@@ -6705,7 +6731,7 @@
         <v>163</v>
       </c>
       <c r="G56" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H56" s="7" t="s">
         <v>38</v>
@@ -6741,7 +6767,7 @@
         <v>2</v>
       </c>
       <c r="Q56" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R56" s="19" t="s">
         <v>11</v>
@@ -6767,7 +6793,7 @@
         <v>165</v>
       </c>
       <c r="G57" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H57" s="7" t="s">
         <v>17</v>
@@ -6803,7 +6829,7 @@
         <v>3</v>
       </c>
       <c r="Q57" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R57" s="19" t="s">
         <v>11</v>
@@ -6829,7 +6855,7 @@
         <v>167</v>
       </c>
       <c r="G58" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H58" s="7" t="s">
         <v>12</v>
@@ -6865,7 +6891,7 @@
         <v>3</v>
       </c>
       <c r="Q58" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R58" s="19" t="s">
         <v>11</v>
@@ -6891,7 +6917,7 @@
         <v>170</v>
       </c>
       <c r="G59" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H59" s="7" t="s">
         <v>23</v>
@@ -6927,7 +6953,7 @@
         <v>3</v>
       </c>
       <c r="Q59" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R59" s="19" t="s">
         <v>11</v>
@@ -6953,7 +6979,7 @@
         <v>173</v>
       </c>
       <c r="G60" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H60" s="7" t="s">
         <v>12</v>
@@ -6989,7 +7015,7 @@
         <v>1</v>
       </c>
       <c r="Q60" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R60" s="19" t="s">
         <v>11</v>
@@ -7006,7 +7032,7 @@
         <v>11</v>
       </c>
       <c r="D61" s="19" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="E61" s="20">
         <v>183</v>
@@ -7015,7 +7041,7 @@
         <v>175</v>
       </c>
       <c r="G61" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H61" s="7" t="s">
         <v>38</v>
@@ -7051,7 +7077,7 @@
         <v>2</v>
       </c>
       <c r="Q61" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R61" s="19" t="s">
         <v>11</v>
@@ -7077,7 +7103,7 @@
         <v>177</v>
       </c>
       <c r="G62" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H62" s="7" t="s">
         <v>12</v>
@@ -7113,7 +7139,7 @@
         <v>2</v>
       </c>
       <c r="Q62" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R62" s="19" t="s">
         <v>11</v>
@@ -7139,10 +7165,10 @@
         <v>179</v>
       </c>
       <c r="G63" s="7" t="s">
+        <v>533</v>
+      </c>
+      <c r="H63" s="7" t="s">
         <v>534</v>
-      </c>
-      <c r="H63" s="7" t="s">
-        <v>535</v>
       </c>
       <c r="I63" s="7">
         <f>VLOOKUP(H63,cardsort_group_IDs!A:B,2,0)</f>
@@ -7175,7 +7201,7 @@
         <v>3</v>
       </c>
       <c r="Q63" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R63" s="19" t="s">
         <v>11</v>
@@ -7192,19 +7218,19 @@
         <v>181</v>
       </c>
       <c r="D64" s="19" t="s">
-        <v>680</v>
+        <v>678</v>
       </c>
       <c r="E64" s="20" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="F64" s="8" t="s">
         <v>182</v>
       </c>
       <c r="G64" s="7" t="s">
+        <v>533</v>
+      </c>
+      <c r="H64" s="7" t="s">
         <v>534</v>
-      </c>
-      <c r="H64" s="7" t="s">
-        <v>535</v>
       </c>
       <c r="I64" s="7">
         <f>VLOOKUP(H64,cardsort_group_IDs!A:B,2,0)</f>
@@ -7257,13 +7283,13 @@
         <v>445</v>
       </c>
       <c r="E65" s="20" t="s">
-        <v>698</v>
+        <v>696</v>
       </c>
       <c r="F65" s="8" t="s">
         <v>184</v>
       </c>
       <c r="G65" s="7" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="H65" s="7" t="s">
         <v>77</v>
@@ -7325,7 +7351,7 @@
         <v>186</v>
       </c>
       <c r="G66" s="7" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="H66" s="7" t="s">
         <v>77</v>
@@ -7361,7 +7387,7 @@
         <v>1</v>
       </c>
       <c r="Q66" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R66" s="19" t="s">
         <v>11</v>
@@ -7387,7 +7413,7 @@
         <v>188</v>
       </c>
       <c r="G67" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H67" s="7" t="s">
         <v>38</v>
@@ -7423,7 +7449,7 @@
         <v>2</v>
       </c>
       <c r="Q67" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R67" s="19" t="s">
         <v>11</v>
@@ -7449,7 +7475,7 @@
         <v>190</v>
       </c>
       <c r="G68" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H68" s="7" t="s">
         <v>12</v>
@@ -7485,7 +7511,7 @@
         <v>1</v>
       </c>
       <c r="Q68" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R68" s="19" t="s">
         <v>11</v>
@@ -7499,10 +7525,10 @@
         <v>191</v>
       </c>
       <c r="C69" s="8" t="s">
-        <v>672</v>
+        <v>670</v>
       </c>
       <c r="D69" s="19" t="s">
-        <v>673</v>
+        <v>671</v>
       </c>
       <c r="E69" s="20" t="s">
         <v>470</v>
@@ -7511,10 +7537,10 @@
         <v>192</v>
       </c>
       <c r="G69" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H69" s="7" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="I69" s="7">
         <f>VLOOKUP(H69,cardsort_group_IDs!A:B,2,0)</f>
@@ -7573,7 +7599,7 @@
         <v>193</v>
       </c>
       <c r="G70" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H70" s="7" t="s">
         <v>23</v>
@@ -7609,7 +7635,7 @@
         <v>2</v>
       </c>
       <c r="Q70" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R70" s="19" t="s">
         <v>11</v>
@@ -7635,7 +7661,7 @@
         <v>195</v>
       </c>
       <c r="G71" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H71" s="7" t="s">
         <v>17</v>
@@ -7671,7 +7697,7 @@
         <v>1</v>
       </c>
       <c r="Q71" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R71" s="19" t="s">
         <v>11</v>
@@ -7691,13 +7717,13 @@
         <v>441</v>
       </c>
       <c r="E72" s="20" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="F72" s="8" t="s">
         <v>197</v>
       </c>
       <c r="G72" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H72" s="7" t="s">
         <v>17</v>
@@ -7733,7 +7759,7 @@
         <v>3</v>
       </c>
       <c r="Q72" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R72" s="19" t="s">
         <v>11</v>
@@ -7750,7 +7776,7 @@
         <v>313</v>
       </c>
       <c r="D73" s="17" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="E73" s="20" t="s">
         <v>433</v>
@@ -7759,7 +7785,7 @@
         <v>199</v>
       </c>
       <c r="G73" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H73" s="7" t="s">
         <v>38</v>
@@ -7795,7 +7821,7 @@
         <v>3</v>
       </c>
       <c r="Q73" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R73" s="19" t="s">
         <v>11</v>
@@ -7821,7 +7847,7 @@
         <v>201</v>
       </c>
       <c r="G74" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H74" s="7" t="s">
         <v>38</v>
@@ -7857,7 +7883,7 @@
         <v>4</v>
       </c>
       <c r="Q74" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R74" s="19" t="s">
         <v>11</v>
@@ -7871,19 +7897,19 @@
         <v>202</v>
       </c>
       <c r="C75" s="8" t="s">
-        <v>665</v>
+        <v>663</v>
       </c>
       <c r="D75" s="19" t="s">
-        <v>666</v>
+        <v>664</v>
       </c>
       <c r="E75" s="20" t="s">
-        <v>699</v>
+        <v>697</v>
       </c>
       <c r="F75" s="8" t="s">
         <v>203</v>
       </c>
       <c r="G75" s="7" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="H75" s="7" t="s">
         <v>38</v>
@@ -7939,13 +7965,13 @@
         <v>441</v>
       </c>
       <c r="E76" s="20" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="F76" s="8" t="s">
         <v>205</v>
       </c>
       <c r="G76" s="7" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="H76" s="7" t="s">
         <v>17</v>
@@ -7981,7 +8007,7 @@
         <v>4</v>
       </c>
       <c r="Q76" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R76" s="19" t="s">
         <v>11</v>
@@ -8007,7 +8033,7 @@
         <v>207</v>
       </c>
       <c r="G77" s="7" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="H77" s="7" t="s">
         <v>54</v>
@@ -8043,7 +8069,7 @@
         <v>3</v>
       </c>
       <c r="Q77" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R77" s="19" t="s">
         <v>11</v>
@@ -8069,7 +8095,7 @@
         <v>209</v>
       </c>
       <c r="G78" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H78" s="7" t="s">
         <v>12</v>
@@ -8105,7 +8131,7 @@
         <v>1</v>
       </c>
       <c r="Q78" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R78" s="19" t="s">
         <v>11</v>
@@ -8131,7 +8157,7 @@
         <v>211</v>
       </c>
       <c r="G79" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H79" s="7" t="s">
         <v>77</v>
@@ -8167,7 +8193,7 @@
         <v>4</v>
       </c>
       <c r="Q79" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R79" s="19" t="s">
         <v>11</v>
@@ -8187,13 +8213,13 @@
         <v>442</v>
       </c>
       <c r="E80" s="20" t="s">
-        <v>590</v>
+        <v>588</v>
       </c>
       <c r="F80" s="8" t="s">
         <v>214</v>
       </c>
       <c r="G80" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H80" s="7" t="s">
         <v>23</v>
@@ -8229,7 +8255,7 @@
         <v>3</v>
       </c>
       <c r="Q80" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R80" s="19" t="s">
         <v>11</v>
@@ -8255,7 +8281,7 @@
         <v>216</v>
       </c>
       <c r="G81" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H81" s="7" t="s">
         <v>23</v>
@@ -8291,7 +8317,7 @@
         <v>1</v>
       </c>
       <c r="Q81" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R81" s="19" t="s">
         <v>11</v>
@@ -8317,7 +8343,7 @@
         <v>218</v>
       </c>
       <c r="G82" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H82" s="7" t="s">
         <v>12</v>
@@ -8353,7 +8379,7 @@
         <v>2</v>
       </c>
       <c r="Q82" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R82" s="19" t="s">
         <v>11</v>
@@ -8379,7 +8405,7 @@
         <v>220</v>
       </c>
       <c r="G83" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H83" s="7" t="s">
         <v>12</v>
@@ -8415,7 +8441,7 @@
         <v>1</v>
       </c>
       <c r="Q83" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R83" s="19" t="s">
         <v>11</v>
@@ -8441,7 +8467,7 @@
         <v>222</v>
       </c>
       <c r="G84" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H84" s="7" t="s">
         <v>12</v>
@@ -8477,7 +8503,7 @@
         <v>1</v>
       </c>
       <c r="Q84" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R84" s="19" t="s">
         <v>11</v>
@@ -8503,7 +8529,7 @@
         <v>225</v>
       </c>
       <c r="G85" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H85" s="7" t="s">
         <v>17</v>
@@ -8539,7 +8565,7 @@
         <v>2</v>
       </c>
       <c r="Q85" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R85" s="19" t="s">
         <v>11</v>
@@ -8565,10 +8591,10 @@
         <v>228</v>
       </c>
       <c r="G86" s="7" t="s">
+        <v>533</v>
+      </c>
+      <c r="H86" s="7" t="s">
         <v>534</v>
-      </c>
-      <c r="H86" s="7" t="s">
-        <v>535</v>
       </c>
       <c r="I86" s="7">
         <f>VLOOKUP(H86,cardsort_group_IDs!A:B,2,0)</f>
@@ -8601,7 +8627,7 @@
         <v>2</v>
       </c>
       <c r="Q86" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R86" s="19" t="s">
         <v>11</v>
@@ -8618,16 +8644,16 @@
         <v>297</v>
       </c>
       <c r="D87" s="20" t="s">
+        <v>559</v>
+      </c>
+      <c r="E87" s="20" t="s">
         <v>560</v>
-      </c>
-      <c r="E87" s="20" t="s">
-        <v>561</v>
       </c>
       <c r="F87" s="8" t="s">
         <v>230</v>
       </c>
       <c r="G87" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H87" s="7" t="s">
         <v>23</v>
@@ -8663,7 +8689,7 @@
         <v>4</v>
       </c>
       <c r="Q87" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R87" s="19" t="s">
         <v>11</v>
@@ -8680,16 +8706,16 @@
         <v>11</v>
       </c>
       <c r="D88" s="19" t="s">
+        <v>543</v>
+      </c>
+      <c r="E88" s="20" t="s">
         <v>544</v>
-      </c>
-      <c r="E88" s="20" t="s">
-        <v>545</v>
       </c>
       <c r="F88" s="8" t="s">
         <v>232</v>
       </c>
       <c r="G88" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H88" s="7" t="s">
         <v>17</v>
@@ -8725,7 +8751,7 @@
         <v>7</v>
       </c>
       <c r="Q88" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R88" s="19" t="s">
         <v>11</v>
@@ -8742,16 +8768,16 @@
         <v>298</v>
       </c>
       <c r="D89" s="19" t="s">
+        <v>567</v>
+      </c>
+      <c r="E89" s="20" t="s">
         <v>568</v>
-      </c>
-      <c r="E89" s="20" t="s">
-        <v>569</v>
       </c>
       <c r="F89" s="8" t="s">
         <v>234</v>
       </c>
       <c r="G89" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H89" s="7" t="s">
         <v>17</v>
@@ -8787,7 +8813,7 @@
         <v>8</v>
       </c>
       <c r="Q89" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R89" s="19" t="s">
         <v>11</v>
@@ -8801,10 +8827,10 @@
         <v>235</v>
       </c>
       <c r="C90" s="8" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="D90" s="20" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="E90" s="20" t="s">
         <v>461</v>
@@ -8813,7 +8839,7 @@
         <v>236</v>
       </c>
       <c r="G90" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H90" s="7" t="s">
         <v>23</v>
@@ -8849,7 +8875,7 @@
         <v>8</v>
       </c>
       <c r="Q90" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R90" s="19" t="s">
         <v>11</v>
@@ -8863,22 +8889,22 @@
         <v>237</v>
       </c>
       <c r="C91" s="8" t="s">
-        <v>11</v>
+        <v>714</v>
       </c>
       <c r="D91" s="19" t="s">
         <v>11</v>
       </c>
-      <c r="E91" s="20">
-        <v>506</v>
+      <c r="E91" s="20" t="s">
+        <v>713</v>
       </c>
       <c r="F91" s="10" t="s">
         <v>238</v>
       </c>
       <c r="G91" s="7" t="s">
+        <v>533</v>
+      </c>
+      <c r="H91" s="7" t="s">
         <v>534</v>
-      </c>
-      <c r="H91" s="7" t="s">
-        <v>535</v>
       </c>
       <c r="I91" s="7">
         <f>VLOOKUP(H91,cardsort_group_IDs!A:B,2,0)</f>
@@ -8904,14 +8930,14 @@
       </c>
       <c r="O91" s="7">
         <f t="shared" si="6"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="P91" s="7">
         <f t="shared" si="7"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q91" s="19" t="s">
-        <v>633</v>
+        <v>136</v>
       </c>
       <c r="R91" s="19" t="s">
         <v>11</v>
@@ -8928,16 +8954,16 @@
         <v>314</v>
       </c>
       <c r="D92" s="17" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="E92" s="20" t="s">
-        <v>570</v>
+        <v>707</v>
       </c>
       <c r="F92" s="8" t="s">
         <v>241</v>
       </c>
       <c r="G92" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H92" s="7" t="s">
         <v>59</v>
@@ -8966,14 +8992,14 @@
       </c>
       <c r="O92" s="7">
         <f t="shared" si="6"/>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="P92" s="7">
         <f t="shared" si="7"/>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="Q92" s="19" t="s">
-        <v>633</v>
+        <v>136</v>
       </c>
       <c r="R92" s="19" t="s">
         <v>11</v>
@@ -8999,7 +9025,7 @@
         <v>243</v>
       </c>
       <c r="G93" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H93" s="7" t="s">
         <v>54</v>
@@ -9035,7 +9061,7 @@
         <v>1</v>
       </c>
       <c r="Q93" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R93" s="19" t="s">
         <v>11</v>
@@ -9061,7 +9087,7 @@
         <v>245</v>
       </c>
       <c r="G94" s="7" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="H94" s="7" t="s">
         <v>38</v>
@@ -9097,7 +9123,7 @@
         <v>4</v>
       </c>
       <c r="Q94" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R94" s="19" t="s">
         <v>11</v>
@@ -9111,7 +9137,7 @@
         <v>43</v>
       </c>
       <c r="C95" s="8" t="s">
-        <v>612</v>
+        <v>610</v>
       </c>
       <c r="D95" s="19" t="s">
         <v>466</v>
@@ -9123,7 +9149,7 @@
         <v>247</v>
       </c>
       <c r="G95" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H95" s="7" t="s">
         <v>38</v>
@@ -9185,7 +9211,7 @@
         <v>249</v>
       </c>
       <c r="G96" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H96" s="7" t="s">
         <v>23</v>
@@ -9221,7 +9247,7 @@
         <v>1</v>
       </c>
       <c r="Q96" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R96" s="19" t="s">
         <v>11</v>
@@ -9247,7 +9273,7 @@
         <v>252</v>
       </c>
       <c r="G97" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H97" s="7" t="s">
         <v>17</v>
@@ -9283,7 +9309,7 @@
         <v>2</v>
       </c>
       <c r="Q97" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R97" s="19" t="s">
         <v>11</v>
@@ -9309,7 +9335,7 @@
         <v>254</v>
       </c>
       <c r="G98" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H98" s="7" t="s">
         <v>17</v>
@@ -9345,7 +9371,7 @@
         <v>3</v>
       </c>
       <c r="Q98" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R98" s="19" t="s">
         <v>11</v>
@@ -9362,7 +9388,7 @@
         <v>315</v>
       </c>
       <c r="D99" s="19" t="s">
-        <v>678</v>
+        <v>676</v>
       </c>
       <c r="E99" s="20" t="s">
         <v>452</v>
@@ -9371,7 +9397,7 @@
         <v>256</v>
       </c>
       <c r="G99" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H99" s="7" t="s">
         <v>17</v>
@@ -9421,19 +9447,19 @@
         <v>257</v>
       </c>
       <c r="C100" s="8" t="s">
-        <v>676</v>
+        <v>674</v>
       </c>
       <c r="D100" s="17" t="s">
-        <v>677</v>
+        <v>675</v>
       </c>
       <c r="E100" s="20" t="s">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="F100" s="8" t="s">
         <v>258</v>
       </c>
       <c r="G100" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H100" s="7" t="s">
         <v>17</v>
@@ -9486,19 +9512,19 @@
         <v>260</v>
       </c>
       <c r="D101" s="19" t="s">
+        <v>545</v>
+      </c>
+      <c r="E101" s="20" t="s">
         <v>546</v>
-      </c>
-      <c r="E101" s="20" t="s">
-        <v>547</v>
       </c>
       <c r="F101" s="8" t="s">
         <v>261</v>
       </c>
       <c r="G101" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H101" s="7" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="I101" s="7">
         <f>VLOOKUP(H101,cardsort_group_IDs!A:B,2,0)</f>
@@ -9531,7 +9557,7 @@
         <v>7</v>
       </c>
       <c r="Q101" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R101" s="19" t="s">
         <v>11</v>
@@ -9557,7 +9583,7 @@
         <v>264</v>
       </c>
       <c r="G102" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H102" s="7" t="s">
         <v>59</v>
@@ -9593,7 +9619,7 @@
         <v>2</v>
       </c>
       <c r="Q102" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R102" s="19" t="s">
         <v>11</v>
@@ -9619,7 +9645,7 @@
         <v>267</v>
       </c>
       <c r="G103" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H103" s="7" t="s">
         <v>59</v>
@@ -9655,7 +9681,7 @@
         <v>3</v>
       </c>
       <c r="Q103" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R103" s="19" t="s">
         <v>11</v>
@@ -9681,7 +9707,7 @@
         <v>269</v>
       </c>
       <c r="G104" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H104" s="7" t="s">
         <v>59</v>
@@ -9717,7 +9743,7 @@
         <v>2</v>
       </c>
       <c r="Q104" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R104" s="19" t="s">
         <v>11</v>
@@ -9728,22 +9754,22 @@
         <v>129</v>
       </c>
       <c r="B105" s="8" t="s">
-        <v>658</v>
+        <v>656</v>
       </c>
       <c r="C105" s="8" t="s">
         <v>302</v>
       </c>
       <c r="D105" s="19" t="s">
-        <v>660</v>
+        <v>658</v>
       </c>
       <c r="E105" s="20" t="s">
-        <v>697</v>
+        <v>695</v>
       </c>
       <c r="F105" s="8" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
       <c r="G105" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H105" s="7" t="s">
         <v>59</v>
@@ -9796,19 +9822,19 @@
         <v>11</v>
       </c>
       <c r="D106" s="19" t="s">
+        <v>547</v>
+      </c>
+      <c r="E106" s="20" t="s">
         <v>548</v>
-      </c>
-      <c r="E106" s="20" t="s">
-        <v>549</v>
       </c>
       <c r="F106" s="8" t="s">
         <v>271</v>
       </c>
       <c r="G106" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H106" s="7" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="I106" s="7">
         <f>VLOOKUP(H106,cardsort_group_IDs!A:B,2,0)</f>
@@ -9841,7 +9867,7 @@
         <v>5</v>
       </c>
       <c r="Q106" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R106" s="19" t="s">
         <v>11</v>
@@ -9858,16 +9884,16 @@
         <v>304</v>
       </c>
       <c r="D107" s="17" t="s">
-        <v>689</v>
+        <v>687</v>
       </c>
       <c r="E107" s="21" t="s">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="F107" s="8" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="G107" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H107" t="s">
         <v>38</v>
@@ -9926,13 +9952,13 @@
         <v>183</v>
       </c>
       <c r="F108" s="8" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="G108" t="s">
+        <v>533</v>
+      </c>
+      <c r="H108" t="s">
         <v>534</v>
-      </c>
-      <c r="H108" t="s">
-        <v>535</v>
       </c>
       <c r="I108" s="7">
         <f>VLOOKUP(H108,cardsort_group_IDs!A:B,2,0)</f>
@@ -9965,7 +9991,7 @@
         <v>1</v>
       </c>
       <c r="Q108" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R108" s="19" t="s">
         <v>11</v>
@@ -9976,7 +10002,7 @@
         <v>136</v>
       </c>
       <c r="B109" s="8" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="C109" s="8" t="s">
         <v>11</v>
@@ -9988,10 +10014,10 @@
         <v>240</v>
       </c>
       <c r="F109" s="8" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="G109" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H109" t="s">
         <v>59</v>
@@ -10027,7 +10053,7 @@
         <v>1</v>
       </c>
       <c r="Q109" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R109" s="19" t="s">
         <v>11</v>
@@ -10050,13 +10076,13 @@
         <v>308</v>
       </c>
       <c r="F110" s="8" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="G110" t="s">
+        <v>533</v>
+      </c>
+      <c r="H110" t="s">
         <v>534</v>
-      </c>
-      <c r="H110" t="s">
-        <v>535</v>
       </c>
       <c r="I110" s="7">
         <f>VLOOKUP(H110,cardsort_group_IDs!A:B,2,0)</f>
@@ -10089,7 +10115,7 @@
         <v>6</v>
       </c>
       <c r="Q110" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R110" s="19" t="s">
         <v>11</v>
@@ -10112,10 +10138,10 @@
         <v>236</v>
       </c>
       <c r="F111" s="15" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="G111" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H111" t="s">
         <v>12</v>
@@ -10151,7 +10177,7 @@
         <v>1</v>
       </c>
       <c r="Q111" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R111" s="19" t="s">
         <v>11</v>
@@ -10162,7 +10188,7 @@
         <v>139</v>
       </c>
       <c r="B112" s="7" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="C112" s="8" t="s">
         <v>11</v>
@@ -10174,10 +10200,10 @@
         <v>11</v>
       </c>
       <c r="F112" s="8" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="G112" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H112" s="7" t="s">
         <v>23</v>
@@ -10213,7 +10239,7 @@
         <v>1</v>
       </c>
       <c r="Q112" s="19" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="R112" s="19" t="s">
         <v>11</v>
@@ -10224,22 +10250,22 @@
         <v>140</v>
       </c>
       <c r="B113" s="7" t="s">
-        <v>622</v>
+        <v>620</v>
       </c>
       <c r="C113" s="8" t="s">
-        <v>653</v>
+        <v>651</v>
       </c>
       <c r="D113" s="19" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="E113" s="20" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
       <c r="F113" s="7" t="s">
-        <v>623</v>
+        <v>621</v>
       </c>
       <c r="G113" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H113" s="7" t="s">
         <v>17</v>
@@ -10275,7 +10301,7 @@
         <v>18</v>
       </c>
       <c r="Q113" s="19" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="R113" s="19">
         <v>2</v>
@@ -10286,22 +10312,22 @@
         <v>141</v>
       </c>
       <c r="B114" s="7" t="s">
+        <v>625</v>
+      </c>
+      <c r="C114" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D114" s="19" t="s">
         <v>627</v>
       </c>
-      <c r="C114" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="D114" s="19" t="s">
-        <v>629</v>
-      </c>
       <c r="E114" s="20" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
       <c r="F114" s="7" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="G114" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H114" s="7" t="s">
         <v>59</v>
@@ -10337,7 +10363,7 @@
         <v>3</v>
       </c>
       <c r="Q114" s="19" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="R114" s="19">
         <v>129</v>
@@ -10348,22 +10374,22 @@
         <v>142</v>
       </c>
       <c r="B115" s="7" t="s">
-        <v>630</v>
+        <v>628</v>
       </c>
       <c r="C115" s="8" t="s">
         <v>11</v>
       </c>
       <c r="D115" s="19" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="E115" s="20" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
       <c r="F115" s="7" t="s">
-        <v>631</v>
+        <v>629</v>
       </c>
       <c r="G115" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H115" s="7" t="s">
         <v>59</v>
@@ -10399,7 +10425,7 @@
         <v>2</v>
       </c>
       <c r="Q115" s="19" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="R115" s="19">
         <v>19</v>
@@ -10410,22 +10436,22 @@
         <v>143</v>
       </c>
       <c r="B116" s="7" t="s">
+        <v>634</v>
+      </c>
+      <c r="C116" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D116" s="19" t="s">
+        <v>635</v>
+      </c>
+      <c r="E116" s="20" t="s">
+        <v>11</v>
+      </c>
+      <c r="F116" s="7" t="s">
         <v>636</v>
       </c>
-      <c r="C116" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="D116" s="19" t="s">
-        <v>637</v>
-      </c>
-      <c r="E116" s="20" t="s">
-        <v>11</v>
-      </c>
-      <c r="F116" s="7" t="s">
-        <v>638</v>
-      </c>
       <c r="G116" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H116" s="7" t="s">
         <v>59</v>
@@ -10461,7 +10487,7 @@
         <v>5</v>
       </c>
       <c r="Q116" s="19" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="R116" s="19" t="s">
         <v>11</v>
@@ -10472,22 +10498,22 @@
         <v>144</v>
       </c>
       <c r="B117" t="s">
-        <v>640</v>
+        <v>638</v>
       </c>
       <c r="C117" s="8" t="s">
         <v>11</v>
       </c>
       <c r="D117" s="17" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="E117" s="20" t="s">
         <v>11</v>
       </c>
       <c r="F117" s="7" t="s">
-        <v>643</v>
+        <v>641</v>
       </c>
       <c r="G117" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H117" s="7" t="s">
         <v>17</v>
@@ -10523,10 +10549,10 @@
         <v>1</v>
       </c>
       <c r="Q117" s="19" t="s">
-        <v>639</v>
+        <v>637</v>
       </c>
       <c r="R117" s="19" t="s">
-        <v>645</v>
+        <v>643</v>
       </c>
     </row>
     <row r="118" spans="1:18" x14ac:dyDescent="0.25">
@@ -10534,22 +10560,22 @@
         <v>145</v>
       </c>
       <c r="B118" s="7" t="s">
+        <v>640</v>
+      </c>
+      <c r="C118" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D118" s="17" t="s">
+        <v>612</v>
+      </c>
+      <c r="E118" s="20" t="s">
+        <v>11</v>
+      </c>
+      <c r="F118" s="7" t="s">
         <v>642</v>
       </c>
-      <c r="C118" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="D118" s="17" t="s">
-        <v>614</v>
-      </c>
-      <c r="E118" s="20" t="s">
-        <v>11</v>
-      </c>
-      <c r="F118" s="7" t="s">
-        <v>644</v>
-      </c>
       <c r="G118" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H118" t="s">
         <v>12</v>
@@ -10585,10 +10611,10 @@
         <v>1</v>
       </c>
       <c r="Q118" s="19" t="s">
-        <v>639</v>
+        <v>637</v>
       </c>
       <c r="R118" s="19" t="s">
-        <v>645</v>
+        <v>643</v>
       </c>
     </row>
     <row r="119" spans="1:18" ht="30" x14ac:dyDescent="0.25">
@@ -10596,22 +10622,22 @@
         <v>146</v>
       </c>
       <c r="B119" s="7" t="s">
-        <v>641</v>
+        <v>639</v>
       </c>
       <c r="C119" s="8" t="s">
-        <v>702</v>
+        <v>700</v>
       </c>
       <c r="D119" t="s">
+        <v>644</v>
+      </c>
+      <c r="E119" s="20" t="s">
+        <v>690</v>
+      </c>
+      <c r="F119" s="7" t="s">
         <v>646</v>
       </c>
-      <c r="E119" s="20" t="s">
-        <v>692</v>
-      </c>
-      <c r="F119" s="7" t="s">
-        <v>648</v>
-      </c>
       <c r="G119" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H119" t="s">
         <v>12</v>
@@ -10647,10 +10673,10 @@
         <v>6</v>
       </c>
       <c r="Q119" s="19" t="s">
-        <v>639</v>
+        <v>637</v>
       </c>
       <c r="R119" s="19" t="s">
-        <v>647</v>
+        <v>645</v>
       </c>
     </row>
     <row r="120" spans="1:18" x14ac:dyDescent="0.25">
@@ -10658,22 +10684,22 @@
         <v>147</v>
       </c>
       <c r="B120" s="7" t="s">
+        <v>647</v>
+      </c>
+      <c r="C120" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D120" s="17" t="s">
         <v>649</v>
       </c>
-      <c r="C120" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="D120" s="17" t="s">
-        <v>651</v>
-      </c>
       <c r="E120" s="20" t="s">
         <v>11</v>
       </c>
       <c r="F120" s="7" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="G120" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H120" s="7" t="s">
         <v>17</v>
@@ -10709,10 +10735,10 @@
         <v>1</v>
       </c>
       <c r="Q120" s="19" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="R120" s="19" t="s">
-        <v>645</v>
+        <v>643</v>
       </c>
     </row>
     <row r="121" spans="1:18" x14ac:dyDescent="0.25">
@@ -10720,22 +10746,22 @@
         <v>148</v>
       </c>
       <c r="B121" s="7" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="C121" s="8" t="s">
-        <v>703</v>
+        <v>701</v>
       </c>
       <c r="D121" t="s">
+        <v>688</v>
+      </c>
+      <c r="E121" s="20" t="s">
         <v>690</v>
       </c>
-      <c r="E121" s="20" t="s">
-        <v>692</v>
-      </c>
       <c r="F121" s="7" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="G121" s="7" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="H121" s="7" t="s">
         <v>12</v>
@@ -10774,7 +10800,7 @@
         <v>136</v>
       </c>
       <c r="R121" s="19" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
     </row>
     <row r="122" spans="1:18" x14ac:dyDescent="0.25">
@@ -10782,22 +10808,22 @@
         <v>149</v>
       </c>
       <c r="B122" s="7" t="s">
-        <v>700</v>
+        <v>698</v>
       </c>
       <c r="C122" s="8" t="s">
         <v>11</v>
       </c>
       <c r="D122" s="19" t="s">
-        <v>679</v>
+        <v>677</v>
       </c>
       <c r="E122" s="20" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
       <c r="F122" s="7" t="s">
-        <v>667</v>
+        <v>665</v>
       </c>
       <c r="G122" s="7" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="H122" s="7" t="s">
         <v>23</v>
@@ -10836,7 +10862,7 @@
         <v>136</v>
       </c>
       <c r="R122" s="19" t="s">
-        <v>668</v>
+        <v>666</v>
       </c>
     </row>
     <row r="123" spans="1:18" x14ac:dyDescent="0.25">
@@ -10844,25 +10870,25 @@
         <v>150</v>
       </c>
       <c r="B123" s="7" t="s">
+        <v>679</v>
+      </c>
+      <c r="C123" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D123" s="19" t="s">
+        <v>680</v>
+      </c>
+      <c r="E123" s="20" t="s">
+        <v>11</v>
+      </c>
+      <c r="F123" s="7" t="s">
         <v>681</v>
       </c>
-      <c r="C123" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="D123" s="19" t="s">
-        <v>682</v>
-      </c>
-      <c r="E123" s="20" t="s">
-        <v>11</v>
-      </c>
-      <c r="F123" s="7" t="s">
-        <v>683</v>
-      </c>
       <c r="G123" s="7" t="s">
+        <v>533</v>
+      </c>
+      <c r="H123" s="7" t="s">
         <v>534</v>
-      </c>
-      <c r="H123" s="7" t="s">
-        <v>535</v>
       </c>
       <c r="I123" s="7">
         <f>VLOOKUP(H123,cardsort_group_IDs!A:B,2,0)</f>
@@ -10898,7 +10924,7 @@
         <v>136</v>
       </c>
       <c r="R123" s="19" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
     </row>
     <row r="124" spans="1:18" ht="30" x14ac:dyDescent="0.25">
@@ -10906,22 +10932,22 @@
         <v>151</v>
       </c>
       <c r="B124" s="7" t="s">
-        <v>694</v>
+        <v>692</v>
       </c>
       <c r="C124" s="8" t="s">
-        <v>704</v>
+        <v>702</v>
       </c>
       <c r="D124" s="19" t="s">
         <v>11</v>
       </c>
       <c r="E124" s="20" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
       <c r="F124" s="7" t="s">
-        <v>695</v>
+        <v>693</v>
       </c>
       <c r="G124" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H124" s="7" t="s">
         <v>17</v>
@@ -10938,37 +10964,216 @@
         <v>327</v>
       </c>
       <c r="L124" s="7">
-        <f t="shared" ref="L124" si="36">IF(E124="-",0,1)+IF(D124="-",0,2)</f>
+        <f t="shared" ref="L124:L125" si="36">IF(E124="-",0,1)+IF(D124="-",0,2)</f>
         <v>1</v>
       </c>
       <c r="M124" s="7">
         <v>10</v>
       </c>
       <c r="N124" s="7">
-        <f t="shared" ref="N124" si="37">IF(D124="-",0,LEN(D124)-LEN(SUBSTITUTE(D124,";",""))+1)</f>
+        <f t="shared" ref="N124:N125" si="37">IF(D124="-",0,LEN(D124)-LEN(SUBSTITUTE(D124,";",""))+1)</f>
         <v>0</v>
       </c>
       <c r="O124" s="7">
-        <f t="shared" ref="O124" si="38">IF(E124="-",0,LEN(E124)-LEN(SUBSTITUTE(E124,";",""))+1)</f>
+        <f t="shared" ref="O124:O125" si="38">IF(E124="-",0,LEN(E124)-LEN(SUBSTITUTE(E124,";",""))+1)</f>
         <v>1</v>
       </c>
       <c r="P124" s="7">
-        <f t="shared" ref="P124" si="39">SUM(N124:O124)</f>
+        <f t="shared" ref="P124:P125" si="39">SUM(N124:O124)</f>
         <v>1</v>
       </c>
       <c r="Q124" s="19" t="s">
         <v>136</v>
       </c>
+      <c r="R124" s="19" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="125" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="N125" s="7"/>
+      <c r="A125" s="7">
+        <v>152</v>
+      </c>
+      <c r="B125" s="7" t="s">
+        <v>708</v>
+      </c>
+      <c r="C125" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D125" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="E125" s="20" t="s">
+        <v>703</v>
+      </c>
+      <c r="F125" s="7" t="s">
+        <v>709</v>
+      </c>
+      <c r="G125" s="7" t="s">
+        <v>533</v>
+      </c>
+      <c r="H125" s="7" t="s">
+        <v>534</v>
+      </c>
+      <c r="I125" s="7">
+        <f>VLOOKUP(H125,cardsort_group_IDs!A:B,2,0)</f>
+        <v>203</v>
+      </c>
+      <c r="J125" s="7" t="s">
+        <v>101</v>
+      </c>
+      <c r="K125" s="7">
+        <f>VLOOKUP(J125,cardsort_subgroup_IDs!A:B,2,0)</f>
+        <v>321</v>
+      </c>
+      <c r="L125" s="7">
+        <f t="shared" ref="L125" si="40">IF(E125="-",0,1)+IF(D125="-",0,2)</f>
+        <v>1</v>
+      </c>
+      <c r="M125" s="7">
+        <v>11</v>
+      </c>
+      <c r="N125" s="7">
+        <f t="shared" ref="N125" si="41">IF(D125="-",0,LEN(D125)-LEN(SUBSTITUTE(D125,";",""))+1)</f>
+        <v>0</v>
+      </c>
+      <c r="O125" s="7">
+        <f t="shared" ref="O125" si="42">IF(E125="-",0,LEN(E125)-LEN(SUBSTITUTE(E125,";",""))+1)</f>
+        <v>1</v>
+      </c>
+      <c r="P125" s="7">
+        <f t="shared" ref="P125" si="43">SUM(N125:O125)</f>
+        <v>1</v>
+      </c>
+      <c r="Q125" s="19" t="s">
+        <v>136</v>
+      </c>
+      <c r="R125" s="19" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="126" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="N126" s="7"/>
+      <c r="A126" s="7">
+        <v>153</v>
+      </c>
+      <c r="B126" s="7" t="s">
+        <v>710</v>
+      </c>
+      <c r="C126" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D126" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="E126" s="20" t="s">
+        <v>703</v>
+      </c>
+      <c r="F126" t="s">
+        <v>712</v>
+      </c>
+      <c r="G126" s="7" t="s">
+        <v>533</v>
+      </c>
+      <c r="H126" s="7" t="s">
+        <v>534</v>
+      </c>
+      <c r="I126" s="7">
+        <f>VLOOKUP(H126,cardsort_group_IDs!A:B,2,0)</f>
+        <v>203</v>
+      </c>
+      <c r="J126" s="7" t="s">
+        <v>104</v>
+      </c>
+      <c r="K126" s="7">
+        <f>VLOOKUP(J126,cardsort_subgroup_IDs!A:B,2,0)</f>
+        <v>322</v>
+      </c>
+      <c r="L126" s="7">
+        <f t="shared" ref="L126" si="44">IF(E126="-",0,1)+IF(D126="-",0,2)</f>
+        <v>1</v>
+      </c>
+      <c r="M126" s="7">
+        <v>12</v>
+      </c>
+      <c r="N126" s="7">
+        <f t="shared" ref="N126" si="45">IF(D126="-",0,LEN(D126)-LEN(SUBSTITUTE(D126,";",""))+1)</f>
+        <v>0</v>
+      </c>
+      <c r="O126" s="7">
+        <f t="shared" ref="O126" si="46">IF(E126="-",0,LEN(E126)-LEN(SUBSTITUTE(E126,";",""))+1)</f>
+        <v>1</v>
+      </c>
+      <c r="P126" s="7">
+        <f t="shared" ref="P126" si="47">SUM(N126:O126)</f>
+        <v>1</v>
+      </c>
+      <c r="Q126" s="19" t="s">
+        <v>136</v>
+      </c>
+      <c r="R126" s="19" t="s">
+        <v>711</v>
+      </c>
     </row>
     <row r="127" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="D127"/>
-      <c r="N127" s="7"/>
+      <c r="A127" s="7">
+        <v>154</v>
+      </c>
+      <c r="B127" s="7" t="s">
+        <v>716</v>
+      </c>
+      <c r="C127" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D127" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="E127" s="20" t="s">
+        <v>703</v>
+      </c>
+      <c r="F127" s="7" t="s">
+        <v>717</v>
+      </c>
+      <c r="G127" s="7" t="s">
+        <v>533</v>
+      </c>
+      <c r="H127" s="7" t="s">
+        <v>534</v>
+      </c>
+      <c r="I127" s="7">
+        <f>VLOOKUP(H127,cardsort_group_IDs!A:B,2,0)</f>
+        <v>203</v>
+      </c>
+      <c r="J127" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="K127" s="7">
+        <f>VLOOKUP(J127,cardsort_subgroup_IDs!A:B,2,0)</f>
+        <v>313</v>
+      </c>
+      <c r="L127" s="7">
+        <f t="shared" ref="L127" si="48">IF(E127="-",0,1)+IF(D127="-",0,2)</f>
+        <v>1</v>
+      </c>
+      <c r="M127" s="7">
+        <v>13</v>
+      </c>
+      <c r="N127" s="7">
+        <f t="shared" ref="N127" si="49">IF(D127="-",0,LEN(D127)-LEN(SUBSTITUTE(D127,";",""))+1)</f>
+        <v>0</v>
+      </c>
+      <c r="O127" s="7">
+        <f t="shared" ref="O127" si="50">IF(E127="-",0,LEN(E127)-LEN(SUBSTITUTE(E127,";",""))+1)</f>
+        <v>1</v>
+      </c>
+      <c r="P127" s="7">
+        <f t="shared" ref="P127" si="51">SUM(N127:O127)</f>
+        <v>1</v>
+      </c>
+      <c r="Q127" s="19" t="s">
+        <v>136</v>
+      </c>
+      <c r="R127" s="19" t="s">
+        <v>715</v>
+      </c>
     </row>
     <row r="128" spans="1:18" x14ac:dyDescent="0.25">
       <c r="N128" s="7"/>
@@ -11120,7 +11325,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{854C4F88-AAAD-435E-8324-B99D91D004B9}">
-  <dimension ref="A1:C134"/>
+  <dimension ref="A1:C135"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="17"/>
@@ -11243,10 +11448,10 @@
         <v>19</v>
       </c>
       <c r="B11" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
       <c r="C11" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -11309,10 +11514,10 @@
         <v>39</v>
       </c>
       <c r="B17" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="C17" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -11452,7 +11657,7 @@
         <v>92</v>
       </c>
       <c r="B30" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="C30" s="15" t="s">
         <v>368</v>
@@ -11595,7 +11800,7 @@
         <v>192</v>
       </c>
       <c r="B43" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="C43" s="15" t="s">
         <v>393</v>
@@ -11606,7 +11811,7 @@
         <v>199</v>
       </c>
       <c r="B44" t="s">
-        <v>624</v>
+        <v>622</v>
       </c>
       <c r="C44" s="15" t="s">
         <v>394</v>
@@ -11639,10 +11844,10 @@
         <v>203</v>
       </c>
       <c r="B47" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="C47" t="s">
-        <v>573</v>
+        <v>571</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
@@ -11664,7 +11869,7 @@
         <v>399</v>
       </c>
       <c r="C49" s="15" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
@@ -11818,7 +12023,7 @@
         <v>274</v>
       </c>
       <c r="C63" s="15" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
@@ -11826,10 +12031,10 @@
         <v>504</v>
       </c>
       <c r="B64" t="s">
+        <v>473</v>
+      </c>
+      <c r="C64" s="15" t="s">
         <v>474</v>
-      </c>
-      <c r="C64" s="15" t="s">
-        <v>475</v>
       </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
@@ -11840,7 +12045,7 @@
         <v>429</v>
       </c>
       <c r="C65" s="15" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
     </row>
     <row r="66" spans="1:3" ht="30" x14ac:dyDescent="0.25">
@@ -11859,7 +12064,7 @@
         <v>507</v>
       </c>
       <c r="B67" t="s">
-        <v>624</v>
+        <v>622</v>
       </c>
       <c r="C67" s="15" t="s">
         <v>431</v>
@@ -11884,7 +12089,7 @@
         <v>139</v>
       </c>
       <c r="C69" s="15" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
     </row>
     <row r="70" spans="1:3" x14ac:dyDescent="0.25">
@@ -11892,18 +12097,18 @@
         <v>510</v>
       </c>
       <c r="B70" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="C70" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71" s="17" t="s">
+        <v>487</v>
+      </c>
+      <c r="B71" t="s">
         <v>488</v>
-      </c>
-      <c r="B71" t="s">
-        <v>489</v>
       </c>
       <c r="C71" s="15" t="s">
         <v>383</v>
@@ -11911,10 +12116,10 @@
     </row>
     <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72" s="17" t="s">
+        <v>489</v>
+      </c>
+      <c r="B72" t="s">
         <v>490</v>
-      </c>
-      <c r="B72" t="s">
-        <v>491</v>
       </c>
       <c r="C72" s="15" t="s">
         <v>383</v>
@@ -11922,10 +12127,10 @@
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73" s="17" t="s">
+        <v>491</v>
+      </c>
+      <c r="B73" t="s">
         <v>492</v>
-      </c>
-      <c r="B73" t="s">
-        <v>493</v>
       </c>
       <c r="C73" s="15" t="s">
         <v>383</v>
@@ -11933,10 +12138,10 @@
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" s="17" t="s">
+        <v>493</v>
+      </c>
+      <c r="B74" t="s">
         <v>494</v>
-      </c>
-      <c r="B74" t="s">
-        <v>495</v>
       </c>
       <c r="C74" s="15" t="s">
         <v>383</v>
@@ -11944,7 +12149,7 @@
     </row>
     <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75" s="17" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="B75" t="s">
         <v>224</v>
@@ -11955,10 +12160,10 @@
     </row>
     <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76" s="17" t="s">
+        <v>496</v>
+      </c>
+      <c r="B76" t="s">
         <v>497</v>
-      </c>
-      <c r="B76" t="s">
-        <v>498</v>
       </c>
       <c r="C76" s="15" t="s">
         <v>383</v>
@@ -11966,10 +12171,10 @@
     </row>
     <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77" s="17" t="s">
+        <v>498</v>
+      </c>
+      <c r="B77" t="s">
         <v>499</v>
-      </c>
-      <c r="B77" t="s">
-        <v>500</v>
       </c>
       <c r="C77" s="15" t="s">
         <v>383</v>
@@ -11977,7 +12182,7 @@
     </row>
     <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78" s="17" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="B78" t="s">
         <v>121</v>
@@ -11988,10 +12193,10 @@
     </row>
     <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79" s="17" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="B79" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C79" s="15" t="s">
         <v>383</v>
@@ -11999,10 +12204,10 @@
     </row>
     <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80" s="17" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="B80" t="s">
-        <v>624</v>
+        <v>622</v>
       </c>
       <c r="C80" s="15" t="s">
         <v>383</v>
@@ -12013,7 +12218,7 @@
         <v>466</v>
       </c>
       <c r="B81" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="C81" s="15" t="s">
         <v>383</v>
@@ -12021,10 +12226,10 @@
     </row>
     <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82" s="17" t="s">
+        <v>504</v>
+      </c>
+      <c r="B82" t="s">
         <v>505</v>
-      </c>
-      <c r="B82" t="s">
-        <v>506</v>
       </c>
       <c r="C82" s="15" t="s">
         <v>383</v>
@@ -12032,10 +12237,10 @@
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" s="17" t="s">
+        <v>506</v>
+      </c>
+      <c r="B83" t="s">
         <v>507</v>
-      </c>
-      <c r="B83" t="s">
-        <v>508</v>
       </c>
       <c r="C83" s="15" t="s">
         <v>383</v>
@@ -12043,10 +12248,10 @@
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" s="17" t="s">
+        <v>508</v>
+      </c>
+      <c r="B84" t="s">
         <v>509</v>
-      </c>
-      <c r="B84" t="s">
-        <v>510</v>
       </c>
       <c r="C84" s="15" t="s">
         <v>383</v>
@@ -12054,7 +12259,7 @@
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85" s="17" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="B85" t="s">
         <v>266</v>
@@ -12065,10 +12270,10 @@
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86" s="17" t="s">
+        <v>511</v>
+      </c>
+      <c r="B86" t="s">
         <v>512</v>
-      </c>
-      <c r="B86" t="s">
-        <v>513</v>
       </c>
       <c r="C86" s="15" t="s">
         <v>383</v>
@@ -12076,10 +12281,10 @@
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87" s="17" t="s">
+        <v>513</v>
+      </c>
+      <c r="B87" t="s">
         <v>514</v>
-      </c>
-      <c r="B87" t="s">
-        <v>515</v>
       </c>
       <c r="C87" s="15" t="s">
         <v>383</v>
@@ -12087,10 +12292,10 @@
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88" s="17" t="s">
+        <v>515</v>
+      </c>
+      <c r="B88" t="s">
         <v>516</v>
-      </c>
-      <c r="B88" t="s">
-        <v>517</v>
       </c>
       <c r="C88" s="15" t="s">
         <v>383</v>
@@ -12098,10 +12303,10 @@
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89" s="17" t="s">
+        <v>517</v>
+      </c>
+      <c r="B89" t="s">
         <v>518</v>
-      </c>
-      <c r="B89" t="s">
-        <v>519</v>
       </c>
       <c r="C89" s="15" t="s">
         <v>383</v>
@@ -12109,10 +12314,10 @@
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A90" s="17" t="s">
+        <v>519</v>
+      </c>
+      <c r="B90" t="s">
         <v>520</v>
-      </c>
-      <c r="B90" t="s">
-        <v>521</v>
       </c>
       <c r="C90" s="15" t="s">
         <v>383</v>
@@ -12120,10 +12325,10 @@
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A91" s="17" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="B91" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="C91" s="15" t="s">
         <v>385</v>
@@ -12131,7 +12336,7 @@
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A92" s="17" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="B92" t="s">
         <v>381</v>
@@ -12142,10 +12347,10 @@
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A93" s="17" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="B93" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="C93" s="15" t="s">
         <v>392</v>
@@ -12164,7 +12369,7 @@
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A95" s="17" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="B95" t="s">
         <v>381</v>
@@ -12175,7 +12380,7 @@
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A96" s="17" t="s">
-        <v>567</v>
+        <v>566</v>
       </c>
       <c r="B96" t="s">
         <v>266</v>
@@ -12186,7 +12391,7 @@
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A97" s="17" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="B97" t="s">
         <v>381</v>
@@ -12197,10 +12402,10 @@
     </row>
     <row r="98" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A98" s="17" t="s">
+        <v>477</v>
+      </c>
+      <c r="B98" t="s">
         <v>478</v>
-      </c>
-      <c r="B98" t="s">
-        <v>479</v>
       </c>
       <c r="C98" s="15" t="s">
         <v>425</v>
@@ -12230,10 +12435,10 @@
     </row>
     <row r="101" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A101" s="17" t="s">
+        <v>479</v>
+      </c>
+      <c r="B101" t="s">
         <v>480</v>
-      </c>
-      <c r="B101" t="s">
-        <v>481</v>
       </c>
       <c r="C101" s="15" t="s">
         <v>425</v>
@@ -12241,10 +12446,10 @@
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A102" s="17" t="s">
+        <v>481</v>
+      </c>
+      <c r="B102" t="s">
         <v>482</v>
-      </c>
-      <c r="B102" t="s">
-        <v>483</v>
       </c>
       <c r="C102" s="15" t="s">
         <v>425</v>
@@ -12252,10 +12457,10 @@
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A103" s="17" t="s">
+        <v>483</v>
+      </c>
+      <c r="B103" t="s">
         <v>484</v>
-      </c>
-      <c r="B103" t="s">
-        <v>485</v>
       </c>
       <c r="C103" s="15" t="s">
         <v>425</v>
@@ -12296,10 +12501,10 @@
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A107" s="17" t="s">
+        <v>485</v>
+      </c>
+      <c r="B107" t="s">
         <v>486</v>
-      </c>
-      <c r="B107" t="s">
-        <v>487</v>
       </c>
       <c r="C107" s="15" t="s">
         <v>425</v>
@@ -12321,7 +12526,7 @@
         <v>445</v>
       </c>
       <c r="B109" t="s">
-        <v>693</v>
+        <v>691</v>
       </c>
       <c r="C109" s="15" t="s">
         <v>425</v>
@@ -12332,7 +12537,7 @@
         <v>446</v>
       </c>
       <c r="B110" t="s">
-        <v>624</v>
+        <v>622</v>
       </c>
       <c r="C110" s="15" t="s">
         <v>425</v>
@@ -12362,7 +12567,7 @@
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A113" s="17" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="B113" t="s">
         <v>381</v>
@@ -12373,7 +12578,7 @@
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A114" s="17" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="B114" t="s">
         <v>381</v>
@@ -12384,222 +12589,233 @@
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A115" s="17" t="s">
-        <v>592</v>
+        <v>590</v>
       </c>
       <c r="B115" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="C115" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A116" s="17" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="B116" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="C116" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A117" s="17" t="s">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="B117" t="s">
         <v>381</v>
       </c>
       <c r="C117" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A118" s="17" t="s">
-        <v>606</v>
+        <v>604</v>
       </c>
       <c r="B118" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="C118" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A119" s="17" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="B119" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="C119" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A120" s="17" t="s">
-        <v>608</v>
+        <v>606</v>
       </c>
       <c r="B120" t="s">
         <v>224</v>
       </c>
       <c r="C120" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A121" s="17" t="s">
-        <v>609</v>
+        <v>607</v>
       </c>
       <c r="B121" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
       <c r="C121" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A122" s="17" t="s">
-        <v>610</v>
+        <v>608</v>
       </c>
       <c r="B122" t="s">
-        <v>597</v>
+        <v>595</v>
       </c>
       <c r="C122" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A123" s="17" t="s">
-        <v>611</v>
+        <v>609</v>
       </c>
       <c r="B123" t="s">
-        <v>621</v>
+        <v>619</v>
       </c>
       <c r="C123" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A124" s="17" t="s">
-        <v>612</v>
+        <v>610</v>
       </c>
       <c r="B124" t="s">
-        <v>598</v>
+        <v>596</v>
       </c>
       <c r="C124" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A125" s="17" t="s">
-        <v>613</v>
+        <v>611</v>
       </c>
       <c r="B125" t="s">
-        <v>599</v>
+        <v>597</v>
       </c>
       <c r="C125" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A126" s="17" t="s">
-        <v>614</v>
+        <v>612</v>
       </c>
       <c r="B126" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="C126" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A127" s="17" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="B127" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="C127" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
     </row>
     <row r="128" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A128" s="17" t="s">
-        <v>616</v>
+        <v>614</v>
       </c>
       <c r="B128" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
       <c r="C128" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
     </row>
     <row r="129" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A129" s="17" t="s">
-        <v>617</v>
+        <v>615</v>
       </c>
       <c r="B129" t="s">
-        <v>603</v>
+        <v>601</v>
       </c>
       <c r="C129" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
     </row>
     <row r="130" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A130" s="17" t="s">
+        <v>616</v>
+      </c>
+      <c r="B130" t="s">
         <v>618</v>
       </c>
-      <c r="B130" t="s">
-        <v>620</v>
-      </c>
       <c r="C130" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
     </row>
     <row r="131" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A131" s="17" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="B131" t="s">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="C131" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A132" s="17" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="B132" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
       <c r="C132" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
     </row>
     <row r="133" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A133" s="17" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
       <c r="B133" t="s">
-        <v>624</v>
+        <v>622</v>
       </c>
       <c r="C133" t="s">
-        <v>591</v>
+        <v>589</v>
       </c>
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A134" s="17" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
       <c r="B134" t="s">
         <v>396</v>
       </c>
       <c r="C134" t="s">
-        <v>691</v>
+        <v>689</v>
+      </c>
+    </row>
+    <row r="135" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A135" s="17" t="s">
+        <v>703</v>
+      </c>
+      <c r="B135" t="s">
+        <v>705</v>
+      </c>
+      <c r="C135" t="s">
+        <v>704</v>
       </c>
     </row>
   </sheetData>
@@ -12638,7 +12854,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="B3">
         <v>203</v>

</xml_diff>

<commit_message>
minor fixes to company naming
</commit_message>
<xml_diff>
--- a/metrics and parser/final_list_of_metrics.xlsx
+++ b/metrics and parser/final_list_of_metrics.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\DATA\DEV\UZH\DX-Metrics-Compass\metrics and parser\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3628999B-BA60-4DEE-BF1A-78C2B5652A9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAACB6FF-1614-4915-ADC8-8F0A32D28403}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="38115" windowHeight="23385" tabRatio="562" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="57840" windowHeight="23520" tabRatio="562" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="metrics" sheetId="1" r:id="rId1"/>
@@ -1753,9 +1753,6 @@
     <t>131l</t>
   </si>
   <si>
-    <t>Facebook (Meta)</t>
-  </si>
-  <si>
     <t>131m</t>
   </si>
   <si>
@@ -2257,9 +2254,6 @@
     <t>Developer CSAT; Developer Experience Index (DXI); Developer Satisfaction Score; Developer Sentiment; Developer Survey with a Focus on Perceptions of Friction; DSAT (Developer Satisfaction); Employee satisfaction; Net User Satisfaction (NSAT); Satisfaction; Satisfaction with Engineering System; Platform and Tool Satisfaction; Developer Ratings for the New System; AI tool CSAT; Bad developer days</t>
   </si>
   <si>
-    <t>501l;  501a;  202a; 501m; 501i; 501f; 501h; 170; 501d; 6a; 510; 511a; 511b; 511d; 511f; 511j; t11k; 511k; 511l; 511n; 511q; 511c; 511e; 511g; 511h; 511m; 511n; 511r</t>
-  </si>
-  <si>
     <t>Time to Release; Feature Delivery Time; Innovation Velocity</t>
   </si>
   <si>
@@ -2390,6 +2384,12 @@
   </si>
   <si>
     <t>Perceived ease and effort to perform a PR.</t>
+  </si>
+  <si>
+    <t>501l;  501a;  202a; 501m; 501i; 501f; 501h; 170; 501d; 6a; 510; 511a; 511b; 511d; 511f; 511j; 511k; 511k; 511l; 511n; 511q; 511c; 511e; 511g; 511h; 511m; 511n; 511r</t>
+  </si>
+  <si>
+    <t>Meta</t>
   </si>
 </sst>
 </file>
@@ -2609,16 +2609,6 @@
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
@@ -2639,21 +2629,21 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF006100"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFC6EFCE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2739,6 +2729,16 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF006100"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF9C5700"/>
       </font>
       <fill>
@@ -2759,21 +2759,21 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C5700"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF006100"/>
       </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
         </patternFill>
       </fill>
     </dxf>
@@ -3348,19 +3348,19 @@
         <v>10</v>
       </c>
       <c r="N1" s="6" t="s">
+        <v>529</v>
+      </c>
+      <c r="O1" s="1" t="s">
         <v>530</v>
       </c>
-      <c r="O1" s="1" t="s">
-        <v>531</v>
-      </c>
       <c r="P1" s="1" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="Q1" s="22" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="R1" s="22" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
     </row>
     <row r="2" spans="1:18" ht="120" x14ac:dyDescent="0.25">
@@ -3374,16 +3374,16 @@
         <v>15</v>
       </c>
       <c r="D2" s="19" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="E2" s="20" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="F2" s="8" t="s">
         <v>16</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H2" s="7" t="s">
         <v>17</v>
@@ -3419,7 +3419,7 @@
         <v>22</v>
       </c>
       <c r="Q2" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R2" s="19" t="s">
         <v>11</v>
@@ -3445,7 +3445,7 @@
         <v>22</v>
       </c>
       <c r="G3" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H3" s="7" t="s">
         <v>23</v>
@@ -3481,7 +3481,7 @@
         <v>1</v>
       </c>
       <c r="Q3" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R3" s="19" t="s">
         <v>11</v>
@@ -3498,19 +3498,19 @@
         <v>275</v>
       </c>
       <c r="D4" s="19" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="E4" s="20" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="F4" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H4" s="7" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="I4" s="7">
         <f>VLOOKUP(H4,cardsort_group_IDs!A:B,2,0)</f>
@@ -3543,7 +3543,7 @@
         <v>8</v>
       </c>
       <c r="Q4" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R4" s="19" t="s">
         <v>11</v>
@@ -3563,13 +3563,13 @@
         <v>485</v>
       </c>
       <c r="E5" s="20" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="F5" s="10" t="s">
         <v>29</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H5" s="7" t="s">
         <v>17</v>
@@ -3605,7 +3605,7 @@
         <v>3</v>
       </c>
       <c r="Q5" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R5" s="19" t="s">
         <v>11</v>
@@ -3625,16 +3625,16 @@
         <v>446</v>
       </c>
       <c r="E6" s="20" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="F6" s="8" t="s">
         <v>32</v>
       </c>
       <c r="G6" s="7" t="s">
+        <v>532</v>
+      </c>
+      <c r="H6" s="7" t="s">
         <v>533</v>
-      </c>
-      <c r="H6" s="7" t="s">
-        <v>534</v>
       </c>
       <c r="I6" s="7">
         <f>VLOOKUP(H6,cardsort_group_IDs!A:B,2,0)</f>
@@ -3667,7 +3667,7 @@
         <v>4</v>
       </c>
       <c r="Q6" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R6" s="19" t="s">
         <v>11</v>
@@ -3693,7 +3693,7 @@
         <v>35</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H7" s="7" t="s">
         <v>12</v>
@@ -3729,7 +3729,7 @@
         <v>1</v>
       </c>
       <c r="Q7" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R7" s="19" t="s">
         <v>11</v>
@@ -3746,16 +3746,16 @@
         <v>11</v>
       </c>
       <c r="D8" s="20" t="s">
-        <v>659</v>
+        <v>658</v>
       </c>
       <c r="E8" s="20" t="s">
-        <v>699</v>
+        <v>697</v>
       </c>
       <c r="F8" s="8" t="s">
         <v>37</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H8" s="7" t="s">
         <v>38</v>
@@ -3817,7 +3817,7 @@
         <v>42</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H9" s="7" t="s">
         <v>38</v>
@@ -3853,7 +3853,7 @@
         <v>1</v>
       </c>
       <c r="Q9" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R9" s="19" t="s">
         <v>11</v>
@@ -3879,7 +3879,7 @@
         <v>45</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H10" s="7" t="s">
         <v>38</v>
@@ -3915,7 +3915,7 @@
         <v>2</v>
       </c>
       <c r="Q10" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R10" s="19" t="s">
         <v>11</v>
@@ -3941,7 +3941,7 @@
         <v>47</v>
       </c>
       <c r="G11" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H11" s="7" t="s">
         <v>17</v>
@@ -3977,7 +3977,7 @@
         <v>3</v>
       </c>
       <c r="Q11" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R11" s="19" t="s">
         <v>11</v>
@@ -4003,7 +4003,7 @@
         <v>49</v>
       </c>
       <c r="G12" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H12" s="7" t="s">
         <v>38</v>
@@ -4039,7 +4039,7 @@
         <v>6</v>
       </c>
       <c r="Q12" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R12" s="19" t="s">
         <v>11</v>
@@ -4056,16 +4056,16 @@
         <v>52</v>
       </c>
       <c r="D13" s="20" t="s">
+        <v>548</v>
+      </c>
+      <c r="E13" s="20" t="s">
         <v>549</v>
-      </c>
-      <c r="E13" s="20" t="s">
-        <v>550</v>
       </c>
       <c r="F13" s="8" t="s">
         <v>53</v>
       </c>
       <c r="G13" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H13" s="7" t="s">
         <v>54</v>
@@ -4101,7 +4101,7 @@
         <v>8</v>
       </c>
       <c r="Q13" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R13" s="19" t="s">
         <v>11</v>
@@ -4115,10 +4115,10 @@
         <v>55</v>
       </c>
       <c r="C14" s="8" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
       <c r="D14" s="19" t="s">
-        <v>685</v>
+        <v>683</v>
       </c>
       <c r="E14" s="20">
         <v>131</v>
@@ -4127,7 +4127,7 @@
         <v>56</v>
       </c>
       <c r="G14" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H14" s="7" t="s">
         <v>38</v>
@@ -4180,16 +4180,16 @@
         <v>277</v>
       </c>
       <c r="D15" s="19" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="E15" s="20" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="F15" s="8" t="s">
         <v>58</v>
       </c>
       <c r="G15" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H15" s="7" t="s">
         <v>59</v>
@@ -4225,7 +4225,7 @@
         <v>26</v>
       </c>
       <c r="Q15" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R15" s="19" t="s">
         <v>11</v>
@@ -4245,16 +4245,16 @@
         <v>11</v>
       </c>
       <c r="E16" s="20" t="s">
-        <v>706</v>
+        <v>704</v>
       </c>
       <c r="F16" s="8" t="s">
         <v>62</v>
       </c>
       <c r="G16" s="7" t="s">
+        <v>532</v>
+      </c>
+      <c r="H16" s="7" t="s">
         <v>533</v>
-      </c>
-      <c r="H16" s="7" t="s">
-        <v>534</v>
       </c>
       <c r="I16" s="7">
         <f>VLOOKUP(H16,cardsort_group_IDs!A:B,2,0)</f>
@@ -4313,7 +4313,7 @@
         <v>66</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H17" s="7" t="s">
         <v>17</v>
@@ -4349,7 +4349,7 @@
         <v>3</v>
       </c>
       <c r="Q17" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R17" s="19" t="s">
         <v>11</v>
@@ -4375,7 +4375,7 @@
         <v>69</v>
       </c>
       <c r="G18" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H18" s="7" t="s">
         <v>54</v>
@@ -4411,7 +4411,7 @@
         <v>2</v>
       </c>
       <c r="Q18" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R18" s="19" t="s">
         <v>11</v>
@@ -4437,7 +4437,7 @@
         <v>73</v>
       </c>
       <c r="G19" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H19" s="7" t="s">
         <v>12</v>
@@ -4473,7 +4473,7 @@
         <v>1</v>
       </c>
       <c r="Q19" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R19" s="19" t="s">
         <v>11</v>
@@ -4493,13 +4493,13 @@
         <v>11</v>
       </c>
       <c r="E20" s="20" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="F20" s="8" t="s">
         <v>76</v>
       </c>
       <c r="G20" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H20" s="7" t="s">
         <v>77</v>
@@ -4535,7 +4535,7 @@
         <v>3</v>
       </c>
       <c r="Q20" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R20" s="19" t="s">
         <v>11</v>
@@ -4561,7 +4561,7 @@
         <v>79</v>
       </c>
       <c r="G21" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H21" s="7" t="s">
         <v>77</v>
@@ -4597,7 +4597,7 @@
         <v>3</v>
       </c>
       <c r="Q21" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R21" s="19" t="s">
         <v>11</v>
@@ -4611,10 +4611,10 @@
         <v>30</v>
       </c>
       <c r="C22" s="8" t="s">
+        <v>660</v>
+      </c>
+      <c r="D22" s="20" t="s">
         <v>661</v>
-      </c>
-      <c r="D22" s="20" t="s">
-        <v>662</v>
       </c>
       <c r="E22" s="20" t="s">
         <v>456</v>
@@ -4623,7 +4623,7 @@
         <v>80</v>
       </c>
       <c r="G22" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H22" s="7" t="s">
         <v>17</v>
@@ -4685,10 +4685,10 @@
         <v>83</v>
       </c>
       <c r="G23" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H23" s="7" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="I23" s="7">
         <f>VLOOKUP(H23,cardsort_group_IDs!A:B,2,0)</f>
@@ -4721,7 +4721,7 @@
         <v>2</v>
       </c>
       <c r="Q23" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R23" s="19" t="s">
         <v>11</v>
@@ -4747,7 +4747,7 @@
         <v>85</v>
       </c>
       <c r="G24" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H24" s="7" t="s">
         <v>38</v>
@@ -4783,7 +4783,7 @@
         <v>1</v>
       </c>
       <c r="Q24" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R24" s="19" t="s">
         <v>11</v>
@@ -4800,16 +4800,16 @@
         <v>11</v>
       </c>
       <c r="D25" s="20" t="s">
-        <v>667</v>
+        <v>666</v>
       </c>
       <c r="E25" s="20" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="F25" s="8" t="s">
         <v>87</v>
       </c>
       <c r="G25" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H25" s="7" t="s">
         <v>77</v>
@@ -4865,13 +4865,13 @@
         <v>170</v>
       </c>
       <c r="E26" s="20" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="F26" s="8" t="s">
         <v>89</v>
       </c>
       <c r="G26" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H26" s="7" t="s">
         <v>38</v>
@@ -4907,7 +4907,7 @@
         <v>4</v>
       </c>
       <c r="Q26" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R26" s="19" t="s">
         <v>11</v>
@@ -4933,7 +4933,7 @@
         <v>93</v>
       </c>
       <c r="G27" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H27" s="7" t="s">
         <v>77</v>
@@ -4969,7 +4969,7 @@
         <v>2</v>
       </c>
       <c r="Q27" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R27" s="19" t="s">
         <v>11</v>
@@ -4995,7 +4995,7 @@
         <v>95</v>
       </c>
       <c r="G28" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H28" s="7" t="s">
         <v>17</v>
@@ -5031,7 +5031,7 @@
         <v>3</v>
       </c>
       <c r="Q28" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R28" s="19" t="s">
         <v>11</v>
@@ -5048,16 +5048,16 @@
         <v>282</v>
       </c>
       <c r="D29" s="20" t="s">
+        <v>550</v>
+      </c>
+      <c r="E29" s="20" t="s">
         <v>551</v>
-      </c>
-      <c r="E29" s="20" t="s">
-        <v>552</v>
       </c>
       <c r="F29" s="8" t="s">
         <v>98</v>
       </c>
       <c r="G29" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H29" s="7" t="s">
         <v>23</v>
@@ -5093,7 +5093,7 @@
         <v>8</v>
       </c>
       <c r="Q29" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R29" s="19" t="s">
         <v>11</v>
@@ -5119,10 +5119,10 @@
         <v>100</v>
       </c>
       <c r="G30" s="7" t="s">
+        <v>532</v>
+      </c>
+      <c r="H30" s="7" t="s">
         <v>533</v>
-      </c>
-      <c r="H30" s="7" t="s">
-        <v>534</v>
       </c>
       <c r="I30" s="7">
         <f>VLOOKUP(H30,cardsort_group_IDs!A:B,2,0)</f>
@@ -5155,7 +5155,7 @@
         <v>3</v>
       </c>
       <c r="Q30" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R30" s="19" t="s">
         <v>11</v>
@@ -5169,22 +5169,22 @@
         <v>102</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
       <c r="D31" s="20" t="s">
-        <v>673</v>
+        <v>716</v>
       </c>
       <c r="E31" s="20" t="s">
-        <v>694</v>
+        <v>692</v>
       </c>
       <c r="F31" s="8" t="s">
         <v>103</v>
       </c>
       <c r="G31" s="7" t="s">
+        <v>532</v>
+      </c>
+      <c r="H31" s="7" t="s">
         <v>533</v>
-      </c>
-      <c r="H31" s="7" t="s">
-        <v>534</v>
       </c>
       <c r="I31" s="7">
         <f>VLOOKUP(H31,cardsort_group_IDs!A:B,2,0)</f>
@@ -5243,7 +5243,7 @@
         <v>106</v>
       </c>
       <c r="G32" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H32" s="7" t="s">
         <v>12</v>
@@ -5279,7 +5279,7 @@
         <v>1</v>
       </c>
       <c r="Q32" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R32" s="19" t="s">
         <v>11</v>
@@ -5296,7 +5296,7 @@
         <v>283</v>
       </c>
       <c r="D33" s="19" t="s">
-        <v>683</v>
+        <v>681</v>
       </c>
       <c r="E33" s="20" t="s">
         <v>468</v>
@@ -5305,7 +5305,7 @@
         <v>108</v>
       </c>
       <c r="G33" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H33" s="7" t="s">
         <v>17</v>
@@ -5367,7 +5367,7 @@
         <v>110</v>
       </c>
       <c r="G34" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H34" s="7" t="s">
         <v>17</v>
@@ -5403,7 +5403,7 @@
         <v>3</v>
       </c>
       <c r="Q34" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R34" s="19" t="s">
         <v>11</v>
@@ -5420,19 +5420,19 @@
         <v>111</v>
       </c>
       <c r="D35" s="20" t="s">
+        <v>540</v>
+      </c>
+      <c r="E35" s="20" t="s">
         <v>541</v>
-      </c>
-      <c r="E35" s="20" t="s">
-        <v>542</v>
       </c>
       <c r="F35" s="8" t="s">
         <v>112</v>
       </c>
       <c r="G35" s="7" t="s">
+        <v>532</v>
+      </c>
+      <c r="H35" s="7" t="s">
         <v>533</v>
-      </c>
-      <c r="H35" s="7" t="s">
-        <v>534</v>
       </c>
       <c r="I35" s="7">
         <f>VLOOKUP(H35,cardsort_group_IDs!A:B,2,0)</f>
@@ -5491,10 +5491,10 @@
         <v>114</v>
       </c>
       <c r="G36" s="7" t="s">
+        <v>532</v>
+      </c>
+      <c r="H36" s="7" t="s">
         <v>533</v>
-      </c>
-      <c r="H36" s="7" t="s">
-        <v>534</v>
       </c>
       <c r="I36" s="7">
         <f>VLOOKUP(H36,cardsort_group_IDs!A:B,2,0)</f>
@@ -5527,7 +5527,7 @@
         <v>6</v>
       </c>
       <c r="Q36" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R36" s="19" t="s">
         <v>11</v>
@@ -5547,13 +5547,13 @@
         <v>11</v>
       </c>
       <c r="E37" s="20" t="s">
-        <v>584</v>
+        <v>583</v>
       </c>
       <c r="F37" s="8" t="s">
         <v>116</v>
       </c>
       <c r="G37" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H37" s="7" t="s">
         <v>38</v>
@@ -5589,7 +5589,7 @@
         <v>2</v>
       </c>
       <c r="Q37" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R37" s="19" t="s">
         <v>11</v>
@@ -5615,10 +5615,10 @@
         <v>118</v>
       </c>
       <c r="G38" s="7" t="s">
+        <v>532</v>
+      </c>
+      <c r="H38" s="7" t="s">
         <v>533</v>
-      </c>
-      <c r="H38" s="7" t="s">
-        <v>534</v>
       </c>
       <c r="I38" s="7">
         <f>VLOOKUP(H38,cardsort_group_IDs!A:B,2,0)</f>
@@ -5651,7 +5651,7 @@
         <v>3</v>
       </c>
       <c r="Q38" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R38" s="19" t="s">
         <v>11</v>
@@ -5665,19 +5665,19 @@
         <v>120</v>
       </c>
       <c r="C39" s="8" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="D39" s="20" t="s">
         <v>442</v>
       </c>
       <c r="E39" s="20" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="F39" s="8" t="s">
         <v>122</v>
       </c>
       <c r="G39" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H39" s="7" t="s">
         <v>23</v>
@@ -5739,7 +5739,7 @@
         <v>125</v>
       </c>
       <c r="G40" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H40" s="7" t="s">
         <v>23</v>
@@ -5775,7 +5775,7 @@
         <v>2</v>
       </c>
       <c r="Q40" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R40" s="19" t="s">
         <v>11</v>
@@ -5801,7 +5801,7 @@
         <v>128</v>
       </c>
       <c r="G41" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H41" s="7" t="s">
         <v>54</v>
@@ -5863,10 +5863,10 @@
         <v>131</v>
       </c>
       <c r="G42" s="7" t="s">
+        <v>532</v>
+      </c>
+      <c r="H42" s="7" t="s">
         <v>533</v>
-      </c>
-      <c r="H42" s="7" t="s">
-        <v>534</v>
       </c>
       <c r="I42" s="7">
         <f>VLOOKUP(H42,cardsort_group_IDs!A:B,2,0)</f>
@@ -5899,7 +5899,7 @@
         <v>2</v>
       </c>
       <c r="Q42" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R42" s="19" t="s">
         <v>11</v>
@@ -5925,7 +5925,7 @@
         <v>133</v>
       </c>
       <c r="G43" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H43" s="7" t="s">
         <v>17</v>
@@ -5961,7 +5961,7 @@
         <v>1</v>
       </c>
       <c r="Q43" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R43" s="19" t="s">
         <v>11</v>
@@ -5987,7 +5987,7 @@
         <v>135</v>
       </c>
       <c r="G44" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H44" s="7" t="s">
         <v>17</v>
@@ -6023,7 +6023,7 @@
         <v>1</v>
       </c>
       <c r="Q44" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R44" s="19" t="s">
         <v>11</v>
@@ -6043,16 +6043,16 @@
         <v>446</v>
       </c>
       <c r="E45" s="20" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="F45" s="8" t="s">
         <v>137</v>
       </c>
       <c r="G45" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H45" s="7" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="I45" s="7">
         <f>VLOOKUP(H45,cardsort_group_IDs!A:B,2,0)</f>
@@ -6085,7 +6085,7 @@
         <v>4</v>
       </c>
       <c r="Q45" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R45" s="19" t="s">
         <v>11</v>
@@ -6111,7 +6111,7 @@
         <v>140</v>
       </c>
       <c r="G46" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H46" s="7" t="s">
         <v>12</v>
@@ -6147,7 +6147,7 @@
         <v>1</v>
       </c>
       <c r="Q46" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R46" s="19" t="s">
         <v>11</v>
@@ -6164,19 +6164,19 @@
         <v>285</v>
       </c>
       <c r="D47" s="19" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="E47" s="20" t="s">
-        <v>583</v>
+        <v>582</v>
       </c>
       <c r="F47" s="8" t="s">
         <v>142</v>
       </c>
       <c r="G47" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H47" s="7" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="I47" s="7">
         <f>VLOOKUP(H47,cardsort_group_IDs!A:B,2,0)</f>
@@ -6235,10 +6235,10 @@
         <v>144</v>
       </c>
       <c r="G48" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H48" s="7" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="I48" s="7">
         <f>VLOOKUP(H48,cardsort_group_IDs!A:B,2,0)</f>
@@ -6288,16 +6288,16 @@
         <v>147</v>
       </c>
       <c r="D49" s="20" t="s">
-        <v>668</v>
+        <v>667</v>
       </c>
       <c r="E49" s="20" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="F49" s="8" t="s">
         <v>148</v>
       </c>
       <c r="G49" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H49" s="7" t="s">
         <v>17</v>
@@ -6333,7 +6333,7 @@
         <v>11</v>
       </c>
       <c r="Q49" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R49" s="19" t="s">
         <v>11</v>
@@ -6350,7 +6350,7 @@
         <v>287</v>
       </c>
       <c r="D50" s="19" t="s">
-        <v>686</v>
+        <v>684</v>
       </c>
       <c r="E50" s="20" t="s">
         <v>465</v>
@@ -6359,7 +6359,7 @@
         <v>151</v>
       </c>
       <c r="G50" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H50" s="7" t="s">
         <v>38</v>
@@ -6421,7 +6421,7 @@
         <v>153</v>
       </c>
       <c r="G51" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H51" s="7" t="s">
         <v>23</v>
@@ -6457,7 +6457,7 @@
         <v>1</v>
       </c>
       <c r="Q51" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R51" s="19" t="s">
         <v>11</v>
@@ -6474,16 +6474,16 @@
         <v>288</v>
       </c>
       <c r="D52" s="20" t="s">
-        <v>669</v>
+        <v>668</v>
       </c>
       <c r="E52" s="20" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="F52" s="8" t="s">
         <v>155</v>
       </c>
       <c r="G52" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H52" s="7" t="s">
         <v>23</v>
@@ -6519,7 +6519,7 @@
         <v>16</v>
       </c>
       <c r="Q52" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R52" s="19" t="s">
         <v>11</v>
@@ -6545,7 +6545,7 @@
         <v>157</v>
       </c>
       <c r="G53" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H53" s="7" t="s">
         <v>54</v>
@@ -6581,7 +6581,7 @@
         <v>1</v>
       </c>
       <c r="Q53" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R53" s="19" t="s">
         <v>11</v>
@@ -6607,7 +6607,7 @@
         <v>159</v>
       </c>
       <c r="G54" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H54" s="7" t="s">
         <v>54</v>
@@ -6643,7 +6643,7 @@
         <v>3</v>
       </c>
       <c r="Q54" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R54" s="19" t="s">
         <v>11</v>
@@ -6669,7 +6669,7 @@
         <v>161</v>
       </c>
       <c r="G55" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H55" s="7" t="s">
         <v>77</v>
@@ -6705,7 +6705,7 @@
         <v>3</v>
       </c>
       <c r="Q55" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R55" s="19" t="s">
         <v>11</v>
@@ -6731,7 +6731,7 @@
         <v>163</v>
       </c>
       <c r="G56" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H56" s="7" t="s">
         <v>38</v>
@@ -6767,7 +6767,7 @@
         <v>2</v>
       </c>
       <c r="Q56" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R56" s="19" t="s">
         <v>11</v>
@@ -6793,7 +6793,7 @@
         <v>165</v>
       </c>
       <c r="G57" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H57" s="7" t="s">
         <v>17</v>
@@ -6829,7 +6829,7 @@
         <v>3</v>
       </c>
       <c r="Q57" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R57" s="19" t="s">
         <v>11</v>
@@ -6855,7 +6855,7 @@
         <v>167</v>
       </c>
       <c r="G58" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H58" s="7" t="s">
         <v>12</v>
@@ -6891,7 +6891,7 @@
         <v>3</v>
       </c>
       <c r="Q58" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R58" s="19" t="s">
         <v>11</v>
@@ -6917,7 +6917,7 @@
         <v>170</v>
       </c>
       <c r="G59" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H59" s="7" t="s">
         <v>23</v>
@@ -6953,7 +6953,7 @@
         <v>3</v>
       </c>
       <c r="Q59" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R59" s="19" t="s">
         <v>11</v>
@@ -6979,7 +6979,7 @@
         <v>173</v>
       </c>
       <c r="G60" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H60" s="7" t="s">
         <v>12</v>
@@ -7015,7 +7015,7 @@
         <v>1</v>
       </c>
       <c r="Q60" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R60" s="19" t="s">
         <v>11</v>
@@ -7032,7 +7032,7 @@
         <v>11</v>
       </c>
       <c r="D61" s="19" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="E61" s="20">
         <v>183</v>
@@ -7041,7 +7041,7 @@
         <v>175</v>
       </c>
       <c r="G61" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H61" s="7" t="s">
         <v>38</v>
@@ -7077,7 +7077,7 @@
         <v>2</v>
       </c>
       <c r="Q61" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R61" s="19" t="s">
         <v>11</v>
@@ -7103,7 +7103,7 @@
         <v>177</v>
       </c>
       <c r="G62" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H62" s="7" t="s">
         <v>12</v>
@@ -7139,7 +7139,7 @@
         <v>2</v>
       </c>
       <c r="Q62" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R62" s="19" t="s">
         <v>11</v>
@@ -7165,10 +7165,10 @@
         <v>179</v>
       </c>
       <c r="G63" s="7" t="s">
+        <v>532</v>
+      </c>
+      <c r="H63" s="7" t="s">
         <v>533</v>
-      </c>
-      <c r="H63" s="7" t="s">
-        <v>534</v>
       </c>
       <c r="I63" s="7">
         <f>VLOOKUP(H63,cardsort_group_IDs!A:B,2,0)</f>
@@ -7201,7 +7201,7 @@
         <v>3</v>
       </c>
       <c r="Q63" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R63" s="19" t="s">
         <v>11</v>
@@ -7218,19 +7218,19 @@
         <v>181</v>
       </c>
       <c r="D64" s="19" t="s">
-        <v>678</v>
+        <v>676</v>
       </c>
       <c r="E64" s="20" t="s">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="F64" s="8" t="s">
         <v>182</v>
       </c>
       <c r="G64" s="7" t="s">
+        <v>532</v>
+      </c>
+      <c r="H64" s="7" t="s">
         <v>533</v>
-      </c>
-      <c r="H64" s="7" t="s">
-        <v>534</v>
       </c>
       <c r="I64" s="7">
         <f>VLOOKUP(H64,cardsort_group_IDs!A:B,2,0)</f>
@@ -7283,13 +7283,13 @@
         <v>445</v>
       </c>
       <c r="E65" s="20" t="s">
-        <v>696</v>
+        <v>694</v>
       </c>
       <c r="F65" s="8" t="s">
         <v>184</v>
       </c>
       <c r="G65" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H65" s="7" t="s">
         <v>77</v>
@@ -7351,7 +7351,7 @@
         <v>186</v>
       </c>
       <c r="G66" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H66" s="7" t="s">
         <v>77</v>
@@ -7387,7 +7387,7 @@
         <v>1</v>
       </c>
       <c r="Q66" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R66" s="19" t="s">
         <v>11</v>
@@ -7413,7 +7413,7 @@
         <v>188</v>
       </c>
       <c r="G67" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H67" s="7" t="s">
         <v>38</v>
@@ -7449,7 +7449,7 @@
         <v>2</v>
       </c>
       <c r="Q67" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R67" s="19" t="s">
         <v>11</v>
@@ -7475,7 +7475,7 @@
         <v>190</v>
       </c>
       <c r="G68" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H68" s="7" t="s">
         <v>12</v>
@@ -7511,7 +7511,7 @@
         <v>1</v>
       </c>
       <c r="Q68" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R68" s="19" t="s">
         <v>11</v>
@@ -7525,10 +7525,10 @@
         <v>191</v>
       </c>
       <c r="C69" s="8" t="s">
+        <v>669</v>
+      </c>
+      <c r="D69" s="19" t="s">
         <v>670</v>
-      </c>
-      <c r="D69" s="19" t="s">
-        <v>671</v>
       </c>
       <c r="E69" s="20" t="s">
         <v>470</v>
@@ -7537,10 +7537,10 @@
         <v>192</v>
       </c>
       <c r="G69" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H69" s="7" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="I69" s="7">
         <f>VLOOKUP(H69,cardsort_group_IDs!A:B,2,0)</f>
@@ -7599,7 +7599,7 @@
         <v>193</v>
       </c>
       <c r="G70" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H70" s="7" t="s">
         <v>23</v>
@@ -7635,7 +7635,7 @@
         <v>2</v>
       </c>
       <c r="Q70" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R70" s="19" t="s">
         <v>11</v>
@@ -7661,7 +7661,7 @@
         <v>195</v>
       </c>
       <c r="G71" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H71" s="7" t="s">
         <v>17</v>
@@ -7697,7 +7697,7 @@
         <v>1</v>
       </c>
       <c r="Q71" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R71" s="19" t="s">
         <v>11</v>
@@ -7717,13 +7717,13 @@
         <v>441</v>
       </c>
       <c r="E72" s="20" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="F72" s="8" t="s">
         <v>197</v>
       </c>
       <c r="G72" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H72" s="7" t="s">
         <v>17</v>
@@ -7759,7 +7759,7 @@
         <v>3</v>
       </c>
       <c r="Q72" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R72" s="19" t="s">
         <v>11</v>
@@ -7776,7 +7776,7 @@
         <v>313</v>
       </c>
       <c r="D73" s="17" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="E73" s="20" t="s">
         <v>433</v>
@@ -7785,7 +7785,7 @@
         <v>199</v>
       </c>
       <c r="G73" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H73" s="7" t="s">
         <v>38</v>
@@ -7821,7 +7821,7 @@
         <v>3</v>
       </c>
       <c r="Q73" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R73" s="19" t="s">
         <v>11</v>
@@ -7847,7 +7847,7 @@
         <v>201</v>
       </c>
       <c r="G74" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H74" s="7" t="s">
         <v>38</v>
@@ -7883,7 +7883,7 @@
         <v>4</v>
       </c>
       <c r="Q74" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R74" s="19" t="s">
         <v>11</v>
@@ -7897,19 +7897,19 @@
         <v>202</v>
       </c>
       <c r="C75" s="8" t="s">
+        <v>662</v>
+      </c>
+      <c r="D75" s="19" t="s">
         <v>663</v>
       </c>
-      <c r="D75" s="19" t="s">
-        <v>664</v>
-      </c>
       <c r="E75" s="20" t="s">
-        <v>697</v>
+        <v>695</v>
       </c>
       <c r="F75" s="8" t="s">
         <v>203</v>
       </c>
       <c r="G75" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H75" s="7" t="s">
         <v>38</v>
@@ -7965,13 +7965,13 @@
         <v>441</v>
       </c>
       <c r="E76" s="20" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="F76" s="8" t="s">
         <v>205</v>
       </c>
       <c r="G76" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H76" s="7" t="s">
         <v>17</v>
@@ -8007,7 +8007,7 @@
         <v>4</v>
       </c>
       <c r="Q76" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R76" s="19" t="s">
         <v>11</v>
@@ -8033,7 +8033,7 @@
         <v>207</v>
       </c>
       <c r="G77" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H77" s="7" t="s">
         <v>54</v>
@@ -8069,7 +8069,7 @@
         <v>3</v>
       </c>
       <c r="Q77" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R77" s="19" t="s">
         <v>11</v>
@@ -8095,7 +8095,7 @@
         <v>209</v>
       </c>
       <c r="G78" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H78" s="7" t="s">
         <v>12</v>
@@ -8131,7 +8131,7 @@
         <v>1</v>
       </c>
       <c r="Q78" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R78" s="19" t="s">
         <v>11</v>
@@ -8157,7 +8157,7 @@
         <v>211</v>
       </c>
       <c r="G79" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H79" s="7" t="s">
         <v>77</v>
@@ -8193,7 +8193,7 @@
         <v>4</v>
       </c>
       <c r="Q79" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R79" s="19" t="s">
         <v>11</v>
@@ -8213,13 +8213,13 @@
         <v>442</v>
       </c>
       <c r="E80" s="20" t="s">
-        <v>588</v>
+        <v>587</v>
       </c>
       <c r="F80" s="8" t="s">
         <v>214</v>
       </c>
       <c r="G80" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H80" s="7" t="s">
         <v>23</v>
@@ -8255,7 +8255,7 @@
         <v>3</v>
       </c>
       <c r="Q80" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R80" s="19" t="s">
         <v>11</v>
@@ -8281,7 +8281,7 @@
         <v>216</v>
       </c>
       <c r="G81" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H81" s="7" t="s">
         <v>23</v>
@@ -8317,7 +8317,7 @@
         <v>1</v>
       </c>
       <c r="Q81" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R81" s="19" t="s">
         <v>11</v>
@@ -8343,7 +8343,7 @@
         <v>218</v>
       </c>
       <c r="G82" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H82" s="7" t="s">
         <v>12</v>
@@ -8379,7 +8379,7 @@
         <v>2</v>
       </c>
       <c r="Q82" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R82" s="19" t="s">
         <v>11</v>
@@ -8405,7 +8405,7 @@
         <v>220</v>
       </c>
       <c r="G83" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H83" s="7" t="s">
         <v>12</v>
@@ -8441,7 +8441,7 @@
         <v>1</v>
       </c>
       <c r="Q83" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R83" s="19" t="s">
         <v>11</v>
@@ -8467,7 +8467,7 @@
         <v>222</v>
       </c>
       <c r="G84" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H84" s="7" t="s">
         <v>12</v>
@@ -8503,7 +8503,7 @@
         <v>1</v>
       </c>
       <c r="Q84" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R84" s="19" t="s">
         <v>11</v>
@@ -8529,7 +8529,7 @@
         <v>225</v>
       </c>
       <c r="G85" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H85" s="7" t="s">
         <v>17</v>
@@ -8565,7 +8565,7 @@
         <v>2</v>
       </c>
       <c r="Q85" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R85" s="19" t="s">
         <v>11</v>
@@ -8591,10 +8591,10 @@
         <v>228</v>
       </c>
       <c r="G86" s="7" t="s">
+        <v>532</v>
+      </c>
+      <c r="H86" s="7" t="s">
         <v>533</v>
-      </c>
-      <c r="H86" s="7" t="s">
-        <v>534</v>
       </c>
       <c r="I86" s="7">
         <f>VLOOKUP(H86,cardsort_group_IDs!A:B,2,0)</f>
@@ -8627,7 +8627,7 @@
         <v>2</v>
       </c>
       <c r="Q86" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R86" s="19" t="s">
         <v>11</v>
@@ -8644,16 +8644,16 @@
         <v>297</v>
       </c>
       <c r="D87" s="20" t="s">
+        <v>558</v>
+      </c>
+      <c r="E87" s="20" t="s">
         <v>559</v>
-      </c>
-      <c r="E87" s="20" t="s">
-        <v>560</v>
       </c>
       <c r="F87" s="8" t="s">
         <v>230</v>
       </c>
       <c r="G87" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H87" s="7" t="s">
         <v>23</v>
@@ -8689,7 +8689,7 @@
         <v>4</v>
       </c>
       <c r="Q87" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R87" s="19" t="s">
         <v>11</v>
@@ -8706,16 +8706,16 @@
         <v>11</v>
       </c>
       <c r="D88" s="19" t="s">
+        <v>542</v>
+      </c>
+      <c r="E88" s="20" t="s">
         <v>543</v>
-      </c>
-      <c r="E88" s="20" t="s">
-        <v>544</v>
       </c>
       <c r="F88" s="8" t="s">
         <v>232</v>
       </c>
       <c r="G88" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H88" s="7" t="s">
         <v>17</v>
@@ -8751,7 +8751,7 @@
         <v>7</v>
       </c>
       <c r="Q88" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R88" s="19" t="s">
         <v>11</v>
@@ -8768,16 +8768,16 @@
         <v>298</v>
       </c>
       <c r="D89" s="19" t="s">
+        <v>566</v>
+      </c>
+      <c r="E89" s="20" t="s">
         <v>567</v>
-      </c>
-      <c r="E89" s="20" t="s">
-        <v>568</v>
       </c>
       <c r="F89" s="8" t="s">
         <v>234</v>
       </c>
       <c r="G89" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H89" s="7" t="s">
         <v>17</v>
@@ -8813,7 +8813,7 @@
         <v>8</v>
       </c>
       <c r="Q89" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R89" s="19" t="s">
         <v>11</v>
@@ -8827,10 +8827,10 @@
         <v>235</v>
       </c>
       <c r="C90" s="8" t="s">
+        <v>576</v>
+      </c>
+      <c r="D90" s="20" t="s">
         <v>577</v>
-      </c>
-      <c r="D90" s="20" t="s">
-        <v>578</v>
       </c>
       <c r="E90" s="20" t="s">
         <v>461</v>
@@ -8839,7 +8839,7 @@
         <v>236</v>
       </c>
       <c r="G90" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H90" s="7" t="s">
         <v>23</v>
@@ -8875,7 +8875,7 @@
         <v>8</v>
       </c>
       <c r="Q90" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R90" s="19" t="s">
         <v>11</v>
@@ -8889,22 +8889,22 @@
         <v>237</v>
       </c>
       <c r="C91" s="8" t="s">
-        <v>714</v>
+        <v>712</v>
       </c>
       <c r="D91" s="19" t="s">
         <v>11</v>
       </c>
       <c r="E91" s="20" t="s">
-        <v>713</v>
+        <v>711</v>
       </c>
       <c r="F91" s="10" t="s">
         <v>238</v>
       </c>
       <c r="G91" s="7" t="s">
+        <v>532</v>
+      </c>
+      <c r="H91" s="7" t="s">
         <v>533</v>
-      </c>
-      <c r="H91" s="7" t="s">
-        <v>534</v>
       </c>
       <c r="I91" s="7">
         <f>VLOOKUP(H91,cardsort_group_IDs!A:B,2,0)</f>
@@ -8954,16 +8954,16 @@
         <v>314</v>
       </c>
       <c r="D92" s="17" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="E92" s="20" t="s">
-        <v>707</v>
+        <v>705</v>
       </c>
       <c r="F92" s="8" t="s">
         <v>241</v>
       </c>
       <c r="G92" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H92" s="7" t="s">
         <v>59</v>
@@ -9025,7 +9025,7 @@
         <v>243</v>
       </c>
       <c r="G93" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H93" s="7" t="s">
         <v>54</v>
@@ -9061,7 +9061,7 @@
         <v>1</v>
       </c>
       <c r="Q93" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R93" s="19" t="s">
         <v>11</v>
@@ -9087,7 +9087,7 @@
         <v>245</v>
       </c>
       <c r="G94" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H94" s="7" t="s">
         <v>38</v>
@@ -9123,7 +9123,7 @@
         <v>4</v>
       </c>
       <c r="Q94" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R94" s="19" t="s">
         <v>11</v>
@@ -9137,7 +9137,7 @@
         <v>43</v>
       </c>
       <c r="C95" s="8" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="D95" s="19" t="s">
         <v>466</v>
@@ -9149,7 +9149,7 @@
         <v>247</v>
       </c>
       <c r="G95" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H95" s="7" t="s">
         <v>38</v>
@@ -9211,7 +9211,7 @@
         <v>249</v>
       </c>
       <c r="G96" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H96" s="7" t="s">
         <v>23</v>
@@ -9247,7 +9247,7 @@
         <v>1</v>
       </c>
       <c r="Q96" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R96" s="19" t="s">
         <v>11</v>
@@ -9273,7 +9273,7 @@
         <v>252</v>
       </c>
       <c r="G97" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H97" s="7" t="s">
         <v>17</v>
@@ -9309,7 +9309,7 @@
         <v>2</v>
       </c>
       <c r="Q97" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R97" s="19" t="s">
         <v>11</v>
@@ -9335,7 +9335,7 @@
         <v>254</v>
       </c>
       <c r="G98" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H98" s="7" t="s">
         <v>17</v>
@@ -9371,7 +9371,7 @@
         <v>3</v>
       </c>
       <c r="Q98" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R98" s="19" t="s">
         <v>11</v>
@@ -9388,7 +9388,7 @@
         <v>315</v>
       </c>
       <c r="D99" s="19" t="s">
-        <v>676</v>
+        <v>674</v>
       </c>
       <c r="E99" s="20" t="s">
         <v>452</v>
@@ -9397,7 +9397,7 @@
         <v>256</v>
       </c>
       <c r="G99" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H99" s="7" t="s">
         <v>17</v>
@@ -9447,19 +9447,19 @@
         <v>257</v>
       </c>
       <c r="C100" s="8" t="s">
-        <v>674</v>
+        <v>672</v>
       </c>
       <c r="D100" s="17" t="s">
-        <v>675</v>
+        <v>673</v>
       </c>
       <c r="E100" s="20" t="s">
-        <v>569</v>
+        <v>568</v>
       </c>
       <c r="F100" s="8" t="s">
         <v>258</v>
       </c>
       <c r="G100" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H100" s="7" t="s">
         <v>17</v>
@@ -9512,19 +9512,19 @@
         <v>260</v>
       </c>
       <c r="D101" s="19" t="s">
+        <v>544</v>
+      </c>
+      <c r="E101" s="20" t="s">
         <v>545</v>
-      </c>
-      <c r="E101" s="20" t="s">
-        <v>546</v>
       </c>
       <c r="F101" s="8" t="s">
         <v>261</v>
       </c>
       <c r="G101" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H101" s="7" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="I101" s="7">
         <f>VLOOKUP(H101,cardsort_group_IDs!A:B,2,0)</f>
@@ -9557,7 +9557,7 @@
         <v>7</v>
       </c>
       <c r="Q101" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R101" s="19" t="s">
         <v>11</v>
@@ -9583,7 +9583,7 @@
         <v>264</v>
       </c>
       <c r="G102" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H102" s="7" t="s">
         <v>59</v>
@@ -9619,7 +9619,7 @@
         <v>2</v>
       </c>
       <c r="Q102" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R102" s="19" t="s">
         <v>11</v>
@@ -9645,7 +9645,7 @@
         <v>267</v>
       </c>
       <c r="G103" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H103" s="7" t="s">
         <v>59</v>
@@ -9681,7 +9681,7 @@
         <v>3</v>
       </c>
       <c r="Q103" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R103" s="19" t="s">
         <v>11</v>
@@ -9707,7 +9707,7 @@
         <v>269</v>
       </c>
       <c r="G104" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H104" s="7" t="s">
         <v>59</v>
@@ -9743,7 +9743,7 @@
         <v>2</v>
       </c>
       <c r="Q104" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R104" s="19" t="s">
         <v>11</v>
@@ -9754,22 +9754,22 @@
         <v>129</v>
       </c>
       <c r="B105" s="8" t="s">
-        <v>656</v>
+        <v>655</v>
       </c>
       <c r="C105" s="8" t="s">
         <v>302</v>
       </c>
       <c r="D105" s="19" t="s">
-        <v>658</v>
+        <v>657</v>
       </c>
       <c r="E105" s="20" t="s">
-        <v>695</v>
+        <v>693</v>
       </c>
       <c r="F105" s="8" t="s">
-        <v>657</v>
+        <v>656</v>
       </c>
       <c r="G105" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H105" s="7" t="s">
         <v>59</v>
@@ -9822,19 +9822,19 @@
         <v>11</v>
       </c>
       <c r="D106" s="19" t="s">
+        <v>546</v>
+      </c>
+      <c r="E106" s="20" t="s">
         <v>547</v>
-      </c>
-      <c r="E106" s="20" t="s">
-        <v>548</v>
       </c>
       <c r="F106" s="8" t="s">
         <v>271</v>
       </c>
       <c r="G106" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H106" s="7" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="I106" s="7">
         <f>VLOOKUP(H106,cardsort_group_IDs!A:B,2,0)</f>
@@ -9867,7 +9867,7 @@
         <v>5</v>
       </c>
       <c r="Q106" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R106" s="19" t="s">
         <v>11</v>
@@ -9884,16 +9884,16 @@
         <v>304</v>
       </c>
       <c r="D107" s="17" t="s">
-        <v>687</v>
+        <v>685</v>
       </c>
       <c r="E107" s="21" t="s">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="F107" s="8" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="G107" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H107" t="s">
         <v>38</v>
@@ -9952,13 +9952,13 @@
         <v>183</v>
       </c>
       <c r="F108" s="8" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="G108" t="s">
+        <v>532</v>
+      </c>
+      <c r="H108" t="s">
         <v>533</v>
-      </c>
-      <c r="H108" t="s">
-        <v>534</v>
       </c>
       <c r="I108" s="7">
         <f>VLOOKUP(H108,cardsort_group_IDs!A:B,2,0)</f>
@@ -9991,7 +9991,7 @@
         <v>1</v>
       </c>
       <c r="Q108" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R108" s="19" t="s">
         <v>11</v>
@@ -10002,7 +10002,7 @@
         <v>136</v>
       </c>
       <c r="B109" s="8" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="C109" s="8" t="s">
         <v>11</v>
@@ -10014,10 +10014,10 @@
         <v>240</v>
       </c>
       <c r="F109" s="8" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="G109" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H109" t="s">
         <v>59</v>
@@ -10053,7 +10053,7 @@
         <v>1</v>
       </c>
       <c r="Q109" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R109" s="19" t="s">
         <v>11</v>
@@ -10076,13 +10076,13 @@
         <v>308</v>
       </c>
       <c r="F110" s="8" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="G110" t="s">
+        <v>532</v>
+      </c>
+      <c r="H110" t="s">
         <v>533</v>
-      </c>
-      <c r="H110" t="s">
-        <v>534</v>
       </c>
       <c r="I110" s="7">
         <f>VLOOKUP(H110,cardsort_group_IDs!A:B,2,0)</f>
@@ -10115,7 +10115,7 @@
         <v>6</v>
       </c>
       <c r="Q110" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R110" s="19" t="s">
         <v>11</v>
@@ -10138,10 +10138,10 @@
         <v>236</v>
       </c>
       <c r="F111" s="15" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="G111" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H111" t="s">
         <v>12</v>
@@ -10177,7 +10177,7 @@
         <v>1</v>
       </c>
       <c r="Q111" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R111" s="19" t="s">
         <v>11</v>
@@ -10188,7 +10188,7 @@
         <v>139</v>
       </c>
       <c r="B112" s="7" t="s">
-        <v>579</v>
+        <v>578</v>
       </c>
       <c r="C112" s="8" t="s">
         <v>11</v>
@@ -10200,10 +10200,10 @@
         <v>11</v>
       </c>
       <c r="F112" s="8" t="s">
-        <v>580</v>
+        <v>579</v>
       </c>
       <c r="G112" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H112" s="7" t="s">
         <v>23</v>
@@ -10239,7 +10239,7 @@
         <v>1</v>
       </c>
       <c r="Q112" s="19" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="R112" s="19" t="s">
         <v>11</v>
@@ -10250,22 +10250,22 @@
         <v>140</v>
       </c>
       <c r="B113" s="7" t="s">
+        <v>619</v>
+      </c>
+      <c r="C113" s="8" t="s">
+        <v>650</v>
+      </c>
+      <c r="D113" s="19" t="s">
+        <v>651</v>
+      </c>
+      <c r="E113" s="20" t="s">
+        <v>688</v>
+      </c>
+      <c r="F113" s="7" t="s">
         <v>620</v>
       </c>
-      <c r="C113" s="8" t="s">
-        <v>651</v>
-      </c>
-      <c r="D113" s="19" t="s">
-        <v>652</v>
-      </c>
-      <c r="E113" s="20" t="s">
-        <v>690</v>
-      </c>
-      <c r="F113" s="7" t="s">
-        <v>621</v>
-      </c>
       <c r="G113" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H113" s="7" t="s">
         <v>17</v>
@@ -10289,7 +10289,7 @@
         <v>0</v>
       </c>
       <c r="N113" s="7">
-        <f t="shared" ref="N113:N114" si="11">IF(D113="-",0,LEN(D113)-LEN(SUBSTITUTE(D113,";",""))+1)</f>
+        <f t="shared" ref="N113" si="11">IF(D113="-",0,LEN(D113)-LEN(SUBSTITUTE(D113,";",""))+1)</f>
         <v>17</v>
       </c>
       <c r="O113" s="7">
@@ -10301,7 +10301,7 @@
         <v>18</v>
       </c>
       <c r="Q113" s="19" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="R113" s="19">
         <v>2</v>
@@ -10312,22 +10312,22 @@
         <v>141</v>
       </c>
       <c r="B114" s="7" t="s">
+        <v>624</v>
+      </c>
+      <c r="C114" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D114" s="19" t="s">
+        <v>626</v>
+      </c>
+      <c r="E114" s="20" t="s">
+        <v>688</v>
+      </c>
+      <c r="F114" s="7" t="s">
         <v>625</v>
       </c>
-      <c r="C114" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="D114" s="19" t="s">
-        <v>627</v>
-      </c>
-      <c r="E114" s="20" t="s">
-        <v>690</v>
-      </c>
-      <c r="F114" s="7" t="s">
-        <v>626</v>
-      </c>
       <c r="G114" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H114" s="7" t="s">
         <v>59</v>
@@ -10351,7 +10351,7 @@
         <v>0</v>
       </c>
       <c r="N114" s="7">
-        <f t="shared" ref="N114:N115" si="12">IF(D114="-",0,LEN(D114)-LEN(SUBSTITUTE(D114,";",""))+1)</f>
+        <f t="shared" ref="N114" si="12">IF(D114="-",0,LEN(D114)-LEN(SUBSTITUTE(D114,";",""))+1)</f>
         <v>2</v>
       </c>
       <c r="O114" s="7">
@@ -10363,7 +10363,7 @@
         <v>3</v>
       </c>
       <c r="Q114" s="19" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="R114" s="19">
         <v>129</v>
@@ -10374,22 +10374,22 @@
         <v>142</v>
       </c>
       <c r="B115" s="7" t="s">
+        <v>627</v>
+      </c>
+      <c r="C115" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D115" s="19" t="s">
+        <v>602</v>
+      </c>
+      <c r="E115" s="20" t="s">
+        <v>688</v>
+      </c>
+      <c r="F115" s="7" t="s">
         <v>628</v>
       </c>
-      <c r="C115" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="D115" s="19" t="s">
-        <v>603</v>
-      </c>
-      <c r="E115" s="20" t="s">
-        <v>690</v>
-      </c>
-      <c r="F115" s="7" t="s">
-        <v>629</v>
-      </c>
       <c r="G115" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H115" s="7" t="s">
         <v>59</v>
@@ -10425,7 +10425,7 @@
         <v>2</v>
       </c>
       <c r="Q115" s="19" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="R115" s="19">
         <v>19</v>
@@ -10436,22 +10436,22 @@
         <v>143</v>
       </c>
       <c r="B116" s="7" t="s">
+        <v>633</v>
+      </c>
+      <c r="C116" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D116" s="19" t="s">
         <v>634</v>
       </c>
-      <c r="C116" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="D116" s="19" t="s">
+      <c r="E116" s="20" t="s">
+        <v>11</v>
+      </c>
+      <c r="F116" s="7" t="s">
         <v>635</v>
       </c>
-      <c r="E116" s="20" t="s">
-        <v>11</v>
-      </c>
-      <c r="F116" s="7" t="s">
-        <v>636</v>
-      </c>
       <c r="G116" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H116" s="7" t="s">
         <v>59</v>
@@ -10487,7 +10487,7 @@
         <v>5</v>
       </c>
       <c r="Q116" s="19" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="R116" s="19" t="s">
         <v>11</v>
@@ -10498,22 +10498,22 @@
         <v>144</v>
       </c>
       <c r="B117" t="s">
-        <v>638</v>
+        <v>637</v>
       </c>
       <c r="C117" s="8" t="s">
         <v>11</v>
       </c>
       <c r="D117" s="17" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="E117" s="20" t="s">
         <v>11</v>
       </c>
       <c r="F117" s="7" t="s">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="G117" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H117" s="7" t="s">
         <v>17</v>
@@ -10549,10 +10549,10 @@
         <v>1</v>
       </c>
       <c r="Q117" s="19" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="R117" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
     </row>
     <row r="118" spans="1:18" x14ac:dyDescent="0.25">
@@ -10560,22 +10560,22 @@
         <v>145</v>
       </c>
       <c r="B118" s="7" t="s">
-        <v>640</v>
+        <v>639</v>
       </c>
       <c r="C118" s="8" t="s">
         <v>11</v>
       </c>
       <c r="D118" s="17" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="E118" s="20" t="s">
         <v>11</v>
       </c>
       <c r="F118" s="7" t="s">
-        <v>642</v>
+        <v>641</v>
       </c>
       <c r="G118" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H118" t="s">
         <v>12</v>
@@ -10592,29 +10592,29 @@
         <v>302</v>
       </c>
       <c r="L118" s="7">
-        <f t="shared" ref="L118:L119" si="16">IF(E118="-",0,1)+IF(D118="-",0,2)</f>
+        <f t="shared" ref="L118" si="16">IF(E118="-",0,1)+IF(D118="-",0,2)</f>
         <v>2</v>
       </c>
       <c r="M118" s="7">
         <v>4</v>
       </c>
       <c r="N118" s="7">
-        <f t="shared" ref="N118:N119" si="17">IF(D118="-",0,LEN(D118)-LEN(SUBSTITUTE(D118,";",""))+1)</f>
+        <f t="shared" ref="N118" si="17">IF(D118="-",0,LEN(D118)-LEN(SUBSTITUTE(D118,";",""))+1)</f>
         <v>1</v>
       </c>
       <c r="O118" s="7">
-        <f t="shared" ref="O118:O119" si="18">IF(E118="-",0,LEN(E118)-LEN(SUBSTITUTE(E118,";",""))+1)</f>
+        <f t="shared" ref="O118" si="18">IF(E118="-",0,LEN(E118)-LEN(SUBSTITUTE(E118,";",""))+1)</f>
         <v>0</v>
       </c>
       <c r="P118" s="7">
-        <f t="shared" ref="P118:P119" si="19">SUM(N118:O118)</f>
+        <f t="shared" ref="P118" si="19">SUM(N118:O118)</f>
         <v>1</v>
       </c>
       <c r="Q118" s="19" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="R118" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
     </row>
     <row r="119" spans="1:18" ht="30" x14ac:dyDescent="0.25">
@@ -10622,22 +10622,22 @@
         <v>146</v>
       </c>
       <c r="B119" s="7" t="s">
-        <v>639</v>
+        <v>638</v>
       </c>
       <c r="C119" s="8" t="s">
-        <v>700</v>
+        <v>698</v>
       </c>
       <c r="D119" t="s">
-        <v>644</v>
+        <v>643</v>
       </c>
       <c r="E119" s="20" t="s">
-        <v>690</v>
+        <v>688</v>
       </c>
       <c r="F119" s="7" t="s">
-        <v>646</v>
+        <v>645</v>
       </c>
       <c r="G119" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H119" t="s">
         <v>12</v>
@@ -10665,18 +10665,18 @@
         <v>5</v>
       </c>
       <c r="O119" s="7">
-        <f t="shared" ref="O119:O122" si="22">IF(E119="-",0,LEN(E119)-LEN(SUBSTITUTE(E119,";",""))+1)</f>
+        <f t="shared" ref="O119:O121" si="22">IF(E119="-",0,LEN(E119)-LEN(SUBSTITUTE(E119,";",""))+1)</f>
         <v>1</v>
       </c>
       <c r="P119" s="7">
-        <f t="shared" ref="P119:P122" si="23">SUM(N119:O119)</f>
+        <f t="shared" ref="P119:P121" si="23">SUM(N119:O119)</f>
         <v>6</v>
       </c>
       <c r="Q119" s="19" t="s">
-        <v>637</v>
+        <v>636</v>
       </c>
       <c r="R119" s="19" t="s">
-        <v>645</v>
+        <v>644</v>
       </c>
     </row>
     <row r="120" spans="1:18" x14ac:dyDescent="0.25">
@@ -10684,22 +10684,22 @@
         <v>147</v>
       </c>
       <c r="B120" s="7" t="s">
+        <v>646</v>
+      </c>
+      <c r="C120" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D120" s="17" t="s">
+        <v>648</v>
+      </c>
+      <c r="E120" s="20" t="s">
+        <v>11</v>
+      </c>
+      <c r="F120" s="7" t="s">
         <v>647</v>
       </c>
-      <c r="C120" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="D120" s="17" t="s">
-        <v>649</v>
-      </c>
-      <c r="E120" s="20" t="s">
-        <v>11</v>
-      </c>
-      <c r="F120" s="7" t="s">
-        <v>648</v>
-      </c>
       <c r="G120" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H120" s="7" t="s">
         <v>17</v>
@@ -10735,10 +10735,10 @@
         <v>1</v>
       </c>
       <c r="Q120" s="19" t="s">
-        <v>623</v>
+        <v>622</v>
       </c>
       <c r="R120" s="19" t="s">
-        <v>643</v>
+        <v>642</v>
       </c>
     </row>
     <row r="121" spans="1:18" x14ac:dyDescent="0.25">
@@ -10746,22 +10746,22 @@
         <v>148</v>
       </c>
       <c r="B121" s="7" t="s">
+        <v>652</v>
+      </c>
+      <c r="C121" s="8" t="s">
+        <v>699</v>
+      </c>
+      <c r="D121" t="s">
+        <v>686</v>
+      </c>
+      <c r="E121" s="20" t="s">
+        <v>688</v>
+      </c>
+      <c r="F121" s="7" t="s">
         <v>653</v>
       </c>
-      <c r="C121" s="8" t="s">
-        <v>701</v>
-      </c>
-      <c r="D121" t="s">
-        <v>688</v>
-      </c>
-      <c r="E121" s="20" t="s">
-        <v>690</v>
-      </c>
-      <c r="F121" s="7" t="s">
-        <v>654</v>
-      </c>
       <c r="G121" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H121" s="7" t="s">
         <v>12</v>
@@ -10778,14 +10778,14 @@
         <v>302</v>
       </c>
       <c r="L121" s="7">
-        <f t="shared" ref="L121:L122" si="26">IF(E121="-",0,1)+IF(D121="-",0,2)</f>
+        <f t="shared" ref="L121" si="26">IF(E121="-",0,1)+IF(D121="-",0,2)</f>
         <v>3</v>
       </c>
       <c r="M121" s="7">
         <v>7</v>
       </c>
       <c r="N121" s="7">
-        <f t="shared" ref="N121:N122" si="27">IF(D121="-",0,LEN(D121)-LEN(SUBSTITUTE(D121,";",""))+1)</f>
+        <f t="shared" ref="N121" si="27">IF(D121="-",0,LEN(D121)-LEN(SUBSTITUTE(D121,";",""))+1)</f>
         <v>10</v>
       </c>
       <c r="O121" s="7">
@@ -10800,7 +10800,7 @@
         <v>136</v>
       </c>
       <c r="R121" s="19" t="s">
-        <v>655</v>
+        <v>654</v>
       </c>
     </row>
     <row r="122" spans="1:18" x14ac:dyDescent="0.25">
@@ -10808,22 +10808,22 @@
         <v>149</v>
       </c>
       <c r="B122" s="7" t="s">
-        <v>698</v>
+        <v>696</v>
       </c>
       <c r="C122" s="8" t="s">
         <v>11</v>
       </c>
       <c r="D122" s="19" t="s">
-        <v>677</v>
+        <v>675</v>
       </c>
       <c r="E122" s="20" t="s">
-        <v>690</v>
+        <v>688</v>
       </c>
       <c r="F122" s="7" t="s">
-        <v>665</v>
+        <v>664</v>
       </c>
       <c r="G122" s="7" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="H122" s="7" t="s">
         <v>23</v>
@@ -10840,7 +10840,7 @@
         <v>304</v>
       </c>
       <c r="L122" s="7">
-        <f t="shared" ref="L122:L123" si="28">IF(E122="-",0,1)+IF(D122="-",0,2)</f>
+        <f t="shared" ref="L122" si="28">IF(E122="-",0,1)+IF(D122="-",0,2)</f>
         <v>3</v>
       </c>
       <c r="M122" s="7">
@@ -10851,7 +10851,7 @@
         <v>2</v>
       </c>
       <c r="O122" s="7">
-        <f t="shared" ref="O122:O123" si="30">IF(E122="-",0,LEN(E122)-LEN(SUBSTITUTE(E122,";",""))+1)</f>
+        <f t="shared" ref="O122" si="30">IF(E122="-",0,LEN(E122)-LEN(SUBSTITUTE(E122,";",""))+1)</f>
         <v>1</v>
       </c>
       <c r="P122" s="7">
@@ -10862,7 +10862,7 @@
         <v>136</v>
       </c>
       <c r="R122" s="19" t="s">
-        <v>666</v>
+        <v>665</v>
       </c>
     </row>
     <row r="123" spans="1:18" x14ac:dyDescent="0.25">
@@ -10870,25 +10870,25 @@
         <v>150</v>
       </c>
       <c r="B123" s="7" t="s">
+        <v>677</v>
+      </c>
+      <c r="C123" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D123" s="19" t="s">
+        <v>678</v>
+      </c>
+      <c r="E123" s="20" t="s">
+        <v>11</v>
+      </c>
+      <c r="F123" s="7" t="s">
         <v>679</v>
       </c>
-      <c r="C123" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="D123" s="19" t="s">
-        <v>680</v>
-      </c>
-      <c r="E123" s="20" t="s">
-        <v>11</v>
-      </c>
-      <c r="F123" s="7" t="s">
-        <v>681</v>
-      </c>
       <c r="G123" s="7" t="s">
+        <v>532</v>
+      </c>
+      <c r="H123" s="7" t="s">
         <v>533</v>
-      </c>
-      <c r="H123" s="7" t="s">
-        <v>534</v>
       </c>
       <c r="I123" s="7">
         <f>VLOOKUP(H123,cardsort_group_IDs!A:B,2,0)</f>
@@ -10902,7 +10902,7 @@
         <v>313</v>
       </c>
       <c r="L123" s="7">
-        <f t="shared" ref="L123:L124" si="32">IF(E123="-",0,1)+IF(D123="-",0,2)</f>
+        <f t="shared" ref="L123" si="32">IF(E123="-",0,1)+IF(D123="-",0,2)</f>
         <v>2</v>
       </c>
       <c r="M123" s="7">
@@ -10913,7 +10913,7 @@
         <v>2</v>
       </c>
       <c r="O123" s="7">
-        <f t="shared" ref="O123:O124" si="34">IF(E123="-",0,LEN(E123)-LEN(SUBSTITUTE(E123,";",""))+1)</f>
+        <f t="shared" ref="O123" si="34">IF(E123="-",0,LEN(E123)-LEN(SUBSTITUTE(E123,";",""))+1)</f>
         <v>0</v>
       </c>
       <c r="P123" s="7">
@@ -10924,7 +10924,7 @@
         <v>136</v>
       </c>
       <c r="R123" s="19" t="s">
-        <v>682</v>
+        <v>680</v>
       </c>
     </row>
     <row r="124" spans="1:18" ht="30" x14ac:dyDescent="0.25">
@@ -10932,22 +10932,22 @@
         <v>151</v>
       </c>
       <c r="B124" s="7" t="s">
-        <v>692</v>
+        <v>690</v>
       </c>
       <c r="C124" s="8" t="s">
-        <v>702</v>
+        <v>700</v>
       </c>
       <c r="D124" s="19" t="s">
         <v>11</v>
       </c>
       <c r="E124" s="20" t="s">
-        <v>690</v>
+        <v>688</v>
       </c>
       <c r="F124" s="7" t="s">
-        <v>693</v>
+        <v>691</v>
       </c>
       <c r="G124" s="7" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="H124" s="7" t="s">
         <v>17</v>
@@ -10964,22 +10964,22 @@
         <v>327</v>
       </c>
       <c r="L124" s="7">
-        <f t="shared" ref="L124:L125" si="36">IF(E124="-",0,1)+IF(D124="-",0,2)</f>
+        <f t="shared" ref="L124" si="36">IF(E124="-",0,1)+IF(D124="-",0,2)</f>
         <v>1</v>
       </c>
       <c r="M124" s="7">
         <v>10</v>
       </c>
       <c r="N124" s="7">
-        <f t="shared" ref="N124:N125" si="37">IF(D124="-",0,LEN(D124)-LEN(SUBSTITUTE(D124,";",""))+1)</f>
+        <f t="shared" ref="N124" si="37">IF(D124="-",0,LEN(D124)-LEN(SUBSTITUTE(D124,";",""))+1)</f>
         <v>0</v>
       </c>
       <c r="O124" s="7">
-        <f t="shared" ref="O124:O125" si="38">IF(E124="-",0,LEN(E124)-LEN(SUBSTITUTE(E124,";",""))+1)</f>
+        <f t="shared" ref="O124" si="38">IF(E124="-",0,LEN(E124)-LEN(SUBSTITUTE(E124,";",""))+1)</f>
         <v>1</v>
       </c>
       <c r="P124" s="7">
-        <f t="shared" ref="P124:P125" si="39">SUM(N124:O124)</f>
+        <f t="shared" ref="P124" si="39">SUM(N124:O124)</f>
         <v>1</v>
       </c>
       <c r="Q124" s="19" t="s">
@@ -10994,7 +10994,7 @@
         <v>152</v>
       </c>
       <c r="B125" s="7" t="s">
-        <v>708</v>
+        <v>706</v>
       </c>
       <c r="C125" s="8" t="s">
         <v>11</v>
@@ -11003,16 +11003,16 @@
         <v>11</v>
       </c>
       <c r="E125" s="20" t="s">
-        <v>703</v>
+        <v>701</v>
       </c>
       <c r="F125" s="7" t="s">
-        <v>709</v>
+        <v>707</v>
       </c>
       <c r="G125" s="7" t="s">
+        <v>532</v>
+      </c>
+      <c r="H125" s="7" t="s">
         <v>533</v>
-      </c>
-      <c r="H125" s="7" t="s">
-        <v>534</v>
       </c>
       <c r="I125" s="7">
         <f>VLOOKUP(H125,cardsort_group_IDs!A:B,2,0)</f>
@@ -11056,25 +11056,25 @@
         <v>153</v>
       </c>
       <c r="B126" s="7" t="s">
+        <v>708</v>
+      </c>
+      <c r="C126" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D126" s="19" t="s">
+        <v>11</v>
+      </c>
+      <c r="E126" s="20" t="s">
+        <v>701</v>
+      </c>
+      <c r="F126" t="s">
         <v>710</v>
       </c>
-      <c r="C126" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="D126" s="19" t="s">
-        <v>11</v>
-      </c>
-      <c r="E126" s="20" t="s">
-        <v>703</v>
-      </c>
-      <c r="F126" t="s">
-        <v>712</v>
-      </c>
       <c r="G126" s="7" t="s">
+        <v>532</v>
+      </c>
+      <c r="H126" s="7" t="s">
         <v>533</v>
-      </c>
-      <c r="H126" s="7" t="s">
-        <v>534</v>
       </c>
       <c r="I126" s="7">
         <f>VLOOKUP(H126,cardsort_group_IDs!A:B,2,0)</f>
@@ -11110,7 +11110,7 @@
         <v>136</v>
       </c>
       <c r="R126" s="19" t="s">
-        <v>711</v>
+        <v>709</v>
       </c>
     </row>
     <row r="127" spans="1:18" x14ac:dyDescent="0.25">
@@ -11118,7 +11118,7 @@
         <v>154</v>
       </c>
       <c r="B127" s="7" t="s">
-        <v>716</v>
+        <v>714</v>
       </c>
       <c r="C127" s="8" t="s">
         <v>11</v>
@@ -11127,16 +11127,16 @@
         <v>11</v>
       </c>
       <c r="E127" s="20" t="s">
-        <v>703</v>
+        <v>701</v>
       </c>
       <c r="F127" s="7" t="s">
-        <v>717</v>
+        <v>715</v>
       </c>
       <c r="G127" s="7" t="s">
+        <v>532</v>
+      </c>
+      <c r="H127" s="7" t="s">
         <v>533</v>
-      </c>
-      <c r="H127" s="7" t="s">
-        <v>534</v>
       </c>
       <c r="I127" s="7">
         <f>VLOOKUP(H127,cardsort_group_IDs!A:B,2,0)</f>
@@ -11172,7 +11172,7 @@
         <v>136</v>
       </c>
       <c r="R127" s="19" t="s">
-        <v>715</v>
+        <v>713</v>
       </c>
     </row>
     <row r="128" spans="1:18" x14ac:dyDescent="0.25">
@@ -11268,54 +11268,54 @@
   <conditionalFormatting sqref="B97">
     <cfRule type="duplicateValues" dxfId="23" priority="3"/>
   </conditionalFormatting>
+  <conditionalFormatting sqref="B112:B116 B119:B1048576">
+    <cfRule type="duplicateValues" dxfId="22" priority="41"/>
+  </conditionalFormatting>
   <conditionalFormatting sqref="F6">
-    <cfRule type="duplicateValues" dxfId="22" priority="26"/>
+    <cfRule type="duplicateValues" dxfId="21" priority="26"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="F36">
-    <cfRule type="duplicateValues" dxfId="21" priority="22"/>
+    <cfRule type="duplicateValues" dxfId="20" priority="22"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="F48">
-    <cfRule type="duplicateValues" dxfId="20" priority="20"/>
     <cfRule type="duplicateValues" dxfId="19" priority="21"/>
+    <cfRule type="duplicateValues" dxfId="18" priority="20"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="F73">
-    <cfRule type="duplicateValues" dxfId="18" priority="7"/>
+    <cfRule type="duplicateValues" dxfId="17" priority="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="F81">
-    <cfRule type="duplicateValues" dxfId="17" priority="8"/>
+    <cfRule type="duplicateValues" dxfId="16" priority="8"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="F87">
-    <cfRule type="duplicateValues" dxfId="16" priority="6"/>
+    <cfRule type="duplicateValues" dxfId="15" priority="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="F100">
-    <cfRule type="duplicateValues" dxfId="15" priority="5"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J16">
-    <cfRule type="duplicateValues" dxfId="14" priority="14"/>
-    <cfRule type="duplicateValues" dxfId="13" priority="15"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="14"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="15"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J35">
-    <cfRule type="duplicateValues" dxfId="12" priority="18"/>
-    <cfRule type="duplicateValues" dxfId="11" priority="19"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="18"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="19"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J47">
-    <cfRule type="duplicateValues" dxfId="10" priority="16"/>
     <cfRule type="duplicateValues" dxfId="9" priority="17"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="16"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J64">
-    <cfRule type="duplicateValues" dxfId="8" priority="12"/>
-    <cfRule type="duplicateValues" dxfId="7" priority="13"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="12"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="13"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J69">
-    <cfRule type="duplicateValues" dxfId="6" priority="10"/>
     <cfRule type="duplicateValues" dxfId="5" priority="11"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="10"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J106">
-    <cfRule type="duplicateValues" dxfId="4" priority="1"/>
     <cfRule type="duplicateValues" dxfId="3" priority="2"/>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B112:B116 B119:B1048576">
-    <cfRule type="duplicateValues" dxfId="2" priority="41"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="1"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -11448,10 +11448,10 @@
         <v>19</v>
       </c>
       <c r="B11" t="s">
-        <v>572</v>
+        <v>571</v>
       </c>
       <c r="C11" t="s">
-        <v>582</v>
+        <v>581</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -11514,10 +11514,10 @@
         <v>39</v>
       </c>
       <c r="B17" t="s">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="C17" t="s">
-        <v>581</v>
+        <v>580</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -11657,7 +11657,7 @@
         <v>92</v>
       </c>
       <c r="B30" t="s">
-        <v>587</v>
+        <v>586</v>
       </c>
       <c r="C30" s="15" t="s">
         <v>368</v>
@@ -11800,7 +11800,7 @@
         <v>192</v>
       </c>
       <c r="B43" t="s">
-        <v>585</v>
+        <v>584</v>
       </c>
       <c r="C43" s="15" t="s">
         <v>393</v>
@@ -11811,7 +11811,7 @@
         <v>199</v>
       </c>
       <c r="B44" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="C44" s="15" t="s">
         <v>394</v>
@@ -11844,10 +11844,10 @@
         <v>203</v>
       </c>
       <c r="B47" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="C47" t="s">
-        <v>571</v>
+        <v>570</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.25">
@@ -11869,7 +11869,7 @@
         <v>399</v>
       </c>
       <c r="C49" s="15" t="s">
-        <v>586</v>
+        <v>585</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
@@ -12064,7 +12064,7 @@
         <v>507</v>
       </c>
       <c r="B67" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="C67" s="15" t="s">
         <v>431</v>
@@ -12097,10 +12097,10 @@
         <v>510</v>
       </c>
       <c r="B70" t="s">
-        <v>576</v>
+        <v>575</v>
       </c>
       <c r="C70" t="s">
-        <v>575</v>
+        <v>574</v>
       </c>
     </row>
     <row r="71" spans="1:3" x14ac:dyDescent="0.25">
@@ -12207,7 +12207,7 @@
         <v>502</v>
       </c>
       <c r="B80" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="C80" s="15" t="s">
         <v>383</v>
@@ -12229,7 +12229,7 @@
         <v>504</v>
       </c>
       <c r="B82" t="s">
-        <v>505</v>
+        <v>717</v>
       </c>
       <c r="C82" s="15" t="s">
         <v>383</v>
@@ -12237,10 +12237,10 @@
     </row>
     <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83" s="17" t="s">
+        <v>505</v>
+      </c>
+      <c r="B83" t="s">
         <v>506</v>
-      </c>
-      <c r="B83" t="s">
-        <v>507</v>
       </c>
       <c r="C83" s="15" t="s">
         <v>383</v>
@@ -12248,10 +12248,10 @@
     </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84" s="17" t="s">
+        <v>507</v>
+      </c>
+      <c r="B84" t="s">
         <v>508</v>
-      </c>
-      <c r="B84" t="s">
-        <v>509</v>
       </c>
       <c r="C84" s="15" t="s">
         <v>383</v>
@@ -12259,7 +12259,7 @@
     </row>
     <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85" s="17" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="B85" t="s">
         <v>266</v>
@@ -12270,10 +12270,10 @@
     </row>
     <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86" s="17" t="s">
+        <v>510</v>
+      </c>
+      <c r="B86" t="s">
         <v>511</v>
-      </c>
-      <c r="B86" t="s">
-        <v>512</v>
       </c>
       <c r="C86" s="15" t="s">
         <v>383</v>
@@ -12281,10 +12281,10 @@
     </row>
     <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87" s="17" t="s">
+        <v>512</v>
+      </c>
+      <c r="B87" t="s">
         <v>513</v>
-      </c>
-      <c r="B87" t="s">
-        <v>514</v>
       </c>
       <c r="C87" s="15" t="s">
         <v>383</v>
@@ -12292,10 +12292,10 @@
     </row>
     <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88" s="17" t="s">
+        <v>514</v>
+      </c>
+      <c r="B88" t="s">
         <v>515</v>
-      </c>
-      <c r="B88" t="s">
-        <v>516</v>
       </c>
       <c r="C88" s="15" t="s">
         <v>383</v>
@@ -12303,10 +12303,10 @@
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89" s="17" t="s">
+        <v>516</v>
+      </c>
+      <c r="B89" t="s">
         <v>517</v>
-      </c>
-      <c r="B89" t="s">
-        <v>518</v>
       </c>
       <c r="C89" s="15" t="s">
         <v>383</v>
@@ -12314,10 +12314,10 @@
     </row>
     <row r="90" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A90" s="17" t="s">
+        <v>518</v>
+      </c>
+      <c r="B90" t="s">
         <v>519</v>
-      </c>
-      <c r="B90" t="s">
-        <v>520</v>
       </c>
       <c r="C90" s="15" t="s">
         <v>383</v>
@@ -12325,10 +12325,10 @@
     </row>
     <row r="91" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A91" s="17" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="B91" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="C91" s="15" t="s">
         <v>385</v>
@@ -12336,7 +12336,7 @@
     </row>
     <row r="92" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A92" s="17" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="B92" t="s">
         <v>381</v>
@@ -12347,7 +12347,7 @@
     </row>
     <row r="93" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A93" s="17" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="B93" t="s">
         <v>503</v>
@@ -12369,7 +12369,7 @@
     </row>
     <row r="95" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A95" s="17" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="B95" t="s">
         <v>381</v>
@@ -12380,7 +12380,7 @@
     </row>
     <row r="96" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A96" s="17" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="B96" t="s">
         <v>266</v>
@@ -12391,7 +12391,7 @@
     </row>
     <row r="97" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A97" s="17" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="B97" t="s">
         <v>381</v>
@@ -12526,7 +12526,7 @@
         <v>445</v>
       </c>
       <c r="B109" t="s">
-        <v>691</v>
+        <v>689</v>
       </c>
       <c r="C109" s="15" t="s">
         <v>425</v>
@@ -12537,7 +12537,7 @@
         <v>446</v>
       </c>
       <c r="B110" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="C110" s="15" t="s">
         <v>425</v>
@@ -12567,7 +12567,7 @@
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A113" s="17" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="B113" t="s">
         <v>381</v>
@@ -12578,7 +12578,7 @@
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A114" s="17" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="B114" t="s">
         <v>381</v>
@@ -12589,233 +12589,233 @@
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A115" s="17" t="s">
+        <v>589</v>
+      </c>
+      <c r="B115" t="s">
         <v>590</v>
       </c>
-      <c r="B115" t="s">
-        <v>591</v>
-      </c>
       <c r="C115" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A116" s="17" t="s">
-        <v>592</v>
+        <v>591</v>
       </c>
       <c r="B116" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="C116" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A117" s="17" t="s">
-        <v>603</v>
+        <v>602</v>
       </c>
       <c r="B117" t="s">
         <v>381</v>
       </c>
       <c r="C117" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A118" s="17" t="s">
-        <v>604</v>
+        <v>603</v>
       </c>
       <c r="B118" t="s">
         <v>488</v>
       </c>
       <c r="C118" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A119" s="17" t="s">
-        <v>605</v>
+        <v>604</v>
       </c>
       <c r="B119" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="C119" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A120" s="17" t="s">
-        <v>606</v>
+        <v>605</v>
       </c>
       <c r="B120" t="s">
         <v>224</v>
       </c>
       <c r="C120" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A121" s="17" t="s">
-        <v>607</v>
+        <v>606</v>
       </c>
       <c r="B121" t="s">
-        <v>594</v>
+        <v>593</v>
       </c>
       <c r="C121" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A122" s="17" t="s">
-        <v>608</v>
+        <v>607</v>
       </c>
       <c r="B122" t="s">
-        <v>595</v>
+        <v>594</v>
       </c>
       <c r="C122" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A123" s="17" t="s">
-        <v>609</v>
+        <v>608</v>
       </c>
       <c r="B123" t="s">
-        <v>619</v>
+        <v>618</v>
       </c>
       <c r="C123" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A124" s="17" t="s">
-        <v>610</v>
+        <v>609</v>
       </c>
       <c r="B124" t="s">
-        <v>596</v>
+        <v>595</v>
       </c>
       <c r="C124" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A125" s="17" t="s">
-        <v>611</v>
+        <v>610</v>
       </c>
       <c r="B125" t="s">
-        <v>597</v>
+        <v>596</v>
       </c>
       <c r="C125" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A126" s="17" t="s">
-        <v>612</v>
+        <v>611</v>
       </c>
       <c r="B126" t="s">
-        <v>598</v>
+        <v>597</v>
       </c>
       <c r="C126" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A127" s="17" t="s">
-        <v>613</v>
+        <v>612</v>
       </c>
       <c r="B127" t="s">
-        <v>599</v>
+        <v>598</v>
       </c>
       <c r="C127" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
     </row>
     <row r="128" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A128" s="17" t="s">
-        <v>614</v>
+        <v>613</v>
       </c>
       <c r="B128" t="s">
-        <v>600</v>
+        <v>599</v>
       </c>
       <c r="C128" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
     </row>
     <row r="129" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A129" s="17" t="s">
-        <v>615</v>
+        <v>614</v>
       </c>
       <c r="B129" t="s">
-        <v>601</v>
+        <v>600</v>
       </c>
       <c r="C129" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
     </row>
     <row r="130" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A130" s="17" t="s">
-        <v>616</v>
+        <v>615</v>
       </c>
       <c r="B130" t="s">
-        <v>618</v>
+        <v>617</v>
       </c>
       <c r="C130" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
     </row>
     <row r="131" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A131" s="17" t="s">
-        <v>617</v>
+        <v>616</v>
       </c>
       <c r="B131" t="s">
-        <v>602</v>
+        <v>601</v>
       </c>
       <c r="C131" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A132" s="17" t="s">
+        <v>648</v>
+      </c>
+      <c r="B132" t="s">
         <v>649</v>
       </c>
-      <c r="B132" t="s">
-        <v>650</v>
-      </c>
       <c r="C132" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
     </row>
     <row r="133" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A133" s="17" t="s">
-        <v>660</v>
+        <v>659</v>
       </c>
       <c r="B133" t="s">
-        <v>622</v>
+        <v>621</v>
       </c>
       <c r="C133" t="s">
-        <v>589</v>
+        <v>588</v>
       </c>
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A134" s="17" t="s">
-        <v>690</v>
+        <v>688</v>
       </c>
       <c r="B134" t="s">
         <v>396</v>
       </c>
       <c r="C134" t="s">
-        <v>689</v>
+        <v>687</v>
       </c>
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A135" s="17" t="s">
+        <v>701</v>
+      </c>
+      <c r="B135" t="s">
         <v>703</v>
       </c>
-      <c r="B135" t="s">
-        <v>705</v>
-      </c>
       <c r="C135" t="s">
-        <v>704</v>
+        <v>702</v>
       </c>
     </row>
   </sheetData>
@@ -12854,7 +12854,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="B3">
         <v>203</v>

</xml_diff>